<commit_message>
printed for subodh sir and migration continue
</commit_message>
<xml_diff>
--- a/2083_2084/estimate/budget maag estimate/Ward swasthya water tank/for prbn.xlsx
+++ b/2083_2084/estimate/budget maag estimate/Ward swasthya water tank/for prbn.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\2083_2084\estimate\budget maag estimate\Ward swasthya water tank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E138D148-A732-49A4-AE28-4B3E6351DC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{042F9B05-4EB5-423A-86B9-20641A921E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'include dhara marmat'!$A$1:$K$173</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'water tank estimate'!$A$1:$K$251</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'water tank estimate'!$A$1:$K$247</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'include dhara marmat'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'water tank estimate'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">WCR!$1:$11</definedName>
@@ -217,7 +217,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="208">
   <si>
     <t>S.N.</t>
   </si>
@@ -791,9 +791,6 @@
     <t>-at wall</t>
   </si>
   <si>
-    <t>Provisional sum for unforseen works at kitchen and water tank</t>
-  </si>
-  <si>
     <t>;'Vvf O{6f 7f8f] 5fKg] sfd</t>
   </si>
   <si>
@@ -806,15 +803,9 @@
     <t>-at cantilever</t>
   </si>
   <si>
-    <t>leQf Pjd\ l;lnËdf @ ld=ld= Kn]g XjfO{6 k'§L Knfi6/ ug]{ sfo{</t>
-  </si>
-  <si>
     <t>-at ward office room 1</t>
   </si>
   <si>
-    <t>- at toilet renovated</t>
-  </si>
-  <si>
     <t>-ceiling</t>
   </si>
   <si>
@@ -824,18 +815,12 @@
     <t>-room 3</t>
   </si>
   <si>
-    <t>Ps sf]6 jf6/ k|'km l;d]G6 sf]6 nufpg] sfd</t>
-  </si>
-  <si>
     <t>-deduction for door</t>
   </si>
   <si>
     <t>-deduction for window</t>
   </si>
   <si>
-    <t>k|fO{d/ afx]s b'O{ sf]6 tof/L jf;]jn l8:6]Dk/ nufpg] sfd .</t>
-  </si>
-  <si>
     <t>-at Ground Floor</t>
   </si>
   <si>
@@ -860,9 +845,6 @@
     <t>-deduction for kitchen rack area</t>
   </si>
   <si>
-    <t>c:t/ jfx]s b'O{ sf]6 j]b/ sf]6 ug]{ sfd</t>
-  </si>
-  <si>
     <t>-at outer face</t>
   </si>
   <si>
@@ -879,6 +861,21 @@
   </si>
   <si>
     <t>Grand Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ;km]{; ;kmf u/L Ps sf]6 k|fO{d/ ;lxt b'O{ sf]6 j]b/sf]6 k]G6 ug]{ sfd</t>
+  </si>
+  <si>
+    <t>;km]{; ;kmf u/L leQf Pjd\ l;lnËdf @ ld=ld= Kn]g XjfO{6 k'§L Knfi6/ ug]{ sfo{</t>
+  </si>
+  <si>
+    <t>;km]{; ;kmf u/L Ps sf]6 jf6/ k|'km l;d]G6 sf]6 nufpg] sfd</t>
+  </si>
+  <si>
+    <t>;km]{; ;kmf u/L Ps sf]6 k|fO{d/ ;lxt b'O{ sf]6 tof/L jf;]jn l8:6]Dk/ nufpg] sfd .</t>
+  </si>
+  <si>
+    <t>Provisional sum for unforseen works at kitchen, water tank and swasthya</t>
   </si>
 </sst>
 </file>
@@ -3171,6 +3168,18 @@
     <xf numFmtId="0" fontId="64" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3187,72 +3196,66 @@
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="61" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="32" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="32" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="61" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="57" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3276,12 +3279,6 @@
     </xf>
     <xf numFmtId="0" fontId="57" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="64" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="64" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="804">
@@ -4497,60 +4494,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="158" t="s">
+      <c r="A1" s="154" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="158"/>
-      <c r="C1" s="158"/>
-      <c r="D1" s="158"/>
-      <c r="E1" s="158"/>
-      <c r="F1" s="158"/>
-      <c r="G1" s="158"/>
-      <c r="H1" s="158"/>
-      <c r="I1" s="158"/>
-      <c r="J1" s="158"/>
+      <c r="B1" s="154"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
+      <c r="I1" s="154"/>
+      <c r="J1" s="154"/>
     </row>
     <row r="2" spans="1:10" ht="25.5">
-      <c r="A2" s="159" t="s">
+      <c r="A2" s="155" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="159"/>
-      <c r="C2" s="159"/>
-      <c r="D2" s="159"/>
-      <c r="E2" s="159"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="159"/>
-      <c r="H2" s="159"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="159"/>
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="155"/>
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="155"/>
     </row>
     <row r="3" spans="1:10" ht="18.75">
-      <c r="A3" s="160" t="s">
+      <c r="A3" s="156" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="160"/>
-      <c r="C3" s="160"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="160"/>
-      <c r="G3" s="160"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="160"/>
-      <c r="J3" s="160"/>
+      <c r="B3" s="156"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="156"/>
+      <c r="F3" s="156"/>
+      <c r="G3" s="156"/>
+      <c r="H3" s="156"/>
+      <c r="I3" s="156"/>
+      <c r="J3" s="156"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="161" t="s">
+      <c r="A4" s="157" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="161"/>
-      <c r="C4" s="161"/>
-      <c r="D4" s="161"/>
-      <c r="E4" s="161"/>
-      <c r="F4" s="161"/>
-      <c r="G4" s="161"/>
-      <c r="H4" s="161"/>
-      <c r="I4" s="161"/>
-      <c r="J4" s="161"/>
+      <c r="B4" s="157"/>
+      <c r="C4" s="157"/>
+      <c r="D4" s="157"/>
+      <c r="E4" s="157"/>
+      <c r="F4" s="157"/>
+      <c r="G4" s="157"/>
+      <c r="H4" s="157"/>
+      <c r="I4" s="157"/>
+      <c r="J4" s="157"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="12"/>
@@ -4569,33 +4566,33 @@
         <v>52</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="162" t="e">
+      <c r="C6" s="158" t="e">
         <f>E51</f>
         <v>#REF!</v>
       </c>
-      <c r="D6" s="163"/>
+      <c r="D6" s="159"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6" t="s">
         <v>53</v>
       </c>
       <c r="H6" s="6"/>
-      <c r="I6" s="162" t="e">
+      <c r="I6" s="158" t="e">
         <f>H51</f>
         <v>#REF!</v>
       </c>
-      <c r="J6" s="163"/>
+      <c r="J6" s="159"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
-      <c r="C7" s="153"/>
-      <c r="D7" s="153"/>
-      <c r="E7" s="153"/>
-      <c r="F7" s="153"/>
-      <c r="H7" s="154"/>
-      <c r="I7" s="154"/>
-      <c r="J7" s="154"/>
+      <c r="C7" s="160"/>
+      <c r="D7" s="160"/>
+      <c r="E7" s="160"/>
+      <c r="F7" s="160"/>
+      <c r="H7" s="161"/>
+      <c r="I7" s="161"/>
+      <c r="J7" s="161"/>
     </row>
     <row r="8" spans="1:10" ht="16.5">
       <c r="A8" t="s">
@@ -4622,32 +4619,32 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="155" t="s">
+      <c r="A10" s="162" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="155" t="s">
+      <c r="B10" s="162" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="157" t="s">
+      <c r="C10" s="164" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="157"/>
-      <c r="E10" s="157"/>
-      <c r="F10" s="157" t="s">
+      <c r="D10" s="164"/>
+      <c r="E10" s="164"/>
+      <c r="F10" s="164" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="157"/>
-      <c r="H10" s="157"/>
-      <c r="I10" s="155" t="s">
+      <c r="G10" s="164"/>
+      <c r="H10" s="164"/>
+      <c r="I10" s="162" t="s">
         <v>60</v>
       </c>
-      <c r="J10" s="155" t="s">
+      <c r="J10" s="162" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="156"/>
-      <c r="B11" s="156"/>
+      <c r="A11" s="163"/>
+      <c r="B11" s="163"/>
       <c r="C11" s="14" t="s">
         <v>61</v>
       </c>
@@ -4666,8 +4663,8 @@
       <c r="H11" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I11" s="156"/>
-      <c r="J11" s="156"/>
+      <c r="I11" s="163"/>
+      <c r="J11" s="163"/>
     </row>
     <row r="12" spans="1:10" ht="15.75">
       <c r="A12" s="22">
@@ -5594,12 +5591,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:J7"/>
@@ -5609,6 +5600,12 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="J10:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -5641,29 +5638,29 @@
       <c r="A1" s="38">
         <v>152</v>
       </c>
-      <c r="B1" s="164" t="s">
+      <c r="B1" s="165" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="165"/>
-      <c r="D1" s="165"/>
-      <c r="E1" s="165"/>
-      <c r="F1" s="165"/>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
+      <c r="C1" s="166"/>
+      <c r="D1" s="166"/>
+      <c r="E1" s="166"/>
+      <c r="F1" s="166"/>
+      <c r="G1" s="166"/>
+      <c r="H1" s="166"/>
     </row>
     <row r="2" spans="1:8" ht="15.75">
       <c r="A2" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="166" t="s">
+      <c r="B2" s="167" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="167"/>
-      <c r="D2" s="167"/>
-      <c r="E2" s="167"/>
-      <c r="F2" s="167"/>
-      <c r="G2" s="167"/>
-      <c r="H2" s="167"/>
+      <c r="C2" s="168"/>
+      <c r="D2" s="168"/>
+      <c r="E2" s="168"/>
+      <c r="F2" s="168"/>
+      <c r="G2" s="168"/>
+      <c r="H2" s="168"/>
     </row>
     <row r="3" spans="1:8" ht="31.5">
       <c r="A3" s="40"/>
@@ -5691,7 +5688,7 @@
     </row>
     <row r="4" spans="1:8" ht="17.25">
       <c r="A4" s="40"/>
-      <c r="B4" s="168" t="s">
+      <c r="B4" s="169" t="s">
         <v>93</v>
       </c>
       <c r="C4" s="42" t="s">
@@ -5714,7 +5711,7 @@
     </row>
     <row r="5" spans="1:8" ht="17.25">
       <c r="A5" s="40"/>
-      <c r="B5" s="169"/>
+      <c r="B5" s="170"/>
       <c r="C5" s="47" t="s">
         <v>96</v>
       </c>
@@ -5738,7 +5735,7 @@
     </row>
     <row r="6" spans="1:8" ht="17.25">
       <c r="A6" s="40"/>
-      <c r="B6" s="170" t="s">
+      <c r="B6" s="171" t="s">
         <v>97</v>
       </c>
       <c r="C6" s="44" t="s">
@@ -5762,7 +5759,7 @@
     </row>
     <row r="7" spans="1:8" ht="17.25">
       <c r="A7" s="40"/>
-      <c r="B7" s="171"/>
+      <c r="B7" s="172"/>
       <c r="C7" s="47" t="s">
         <v>100</v>
       </c>
@@ -5887,94 +5884,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="150" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="146"/>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="150"/>
       <c r="L1" s="109"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="147" t="s">
+      <c r="A2" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="147"/>
-      <c r="C2" s="147"/>
-      <c r="D2" s="147"/>
-      <c r="E2" s="147"/>
-      <c r="F2" s="147"/>
-      <c r="G2" s="147"/>
-      <c r="H2" s="147"/>
-      <c r="I2" s="147"/>
-      <c r="J2" s="147"/>
-      <c r="K2" s="147"/>
+      <c r="B2" s="151"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="151"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="151"/>
+      <c r="H2" s="151"/>
+      <c r="I2" s="151"/>
+      <c r="J2" s="151"/>
+      <c r="K2" s="151"/>
       <c r="L2" s="118"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="146" t="s">
+      <c r="A3" s="150" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="146"/>
-      <c r="C3" s="146"/>
-      <c r="D3" s="146"/>
-      <c r="E3" s="146"/>
-      <c r="F3" s="146"/>
-      <c r="G3" s="146"/>
-      <c r="H3" s="146"/>
-      <c r="I3" s="146"/>
-      <c r="J3" s="146"/>
-      <c r="K3" s="146"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="150"/>
+      <c r="D3" s="150"/>
+      <c r="E3" s="150"/>
+      <c r="F3" s="150"/>
+      <c r="G3" s="150"/>
+      <c r="H3" s="150"/>
+      <c r="I3" s="150"/>
+      <c r="J3" s="150"/>
+      <c r="K3" s="150"/>
       <c r="L3" s="109"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="148" t="s">
+      <c r="A4" s="152" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="148"/>
-      <c r="C4" s="148"/>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
-      <c r="F4" s="148"/>
-      <c r="G4" s="148"/>
-      <c r="H4" s="148"/>
-      <c r="I4" s="148"/>
-      <c r="J4" s="148"/>
-      <c r="K4" s="148"/>
+      <c r="B4" s="152"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
+      <c r="F4" s="152"/>
+      <c r="G4" s="152"/>
+      <c r="H4" s="152"/>
+      <c r="I4" s="152"/>
+      <c r="J4" s="152"/>
+      <c r="K4" s="152"/>
     </row>
     <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="119" t="s">
         <v>139</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="J5" s="149" t="s">
+      <c r="J5" s="153" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="149"/>
+      <c r="K5" s="153"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="144" t="s">
+      <c r="A6" s="148" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="144"/>
-      <c r="C6" s="144"/>
-      <c r="D6" s="144"/>
-      <c r="E6" s="144"/>
-      <c r="F6" s="144"/>
+      <c r="B6" s="148"/>
+      <c r="C6" s="148"/>
+      <c r="D6" s="148"/>
+      <c r="E6" s="148"/>
+      <c r="F6" s="148"/>
       <c r="G6" s="61"/>
-      <c r="H6" s="145" t="s">
+      <c r="H6" s="149" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="145"/>
-      <c r="J6" s="145"/>
-      <c r="K6" s="145"/>
+      <c r="I6" s="149"/>
+      <c r="J6" s="149"/>
+      <c r="K6" s="149"/>
     </row>
     <row r="7" spans="1:12">
       <c r="B7" s="3"/>
@@ -9323,10 +9320,10 @@
       <c r="B167" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C167" s="151" t="s">
+      <c r="C167" s="144" t="s">
         <v>66</v>
       </c>
-      <c r="D167" s="151"/>
+      <c r="D167" s="144"/>
       <c r="E167" s="75" t="s">
         <v>67</v>
       </c>
@@ -9342,11 +9339,11 @@
       <c r="B168" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="C168" s="152">
+      <c r="C168" s="145">
         <f>+J165</f>
         <v>530004.91742540663</v>
       </c>
-      <c r="D168" s="152"/>
+      <c r="D168" s="145"/>
       <c r="E168" s="110"/>
       <c r="F168" s="108"/>
       <c r="G168" s="111"/>
@@ -9360,10 +9357,10 @@
       <c r="B169" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="C169" s="152">
+      <c r="C169" s="145">
         <v>480000</v>
       </c>
-      <c r="D169" s="152"/>
+      <c r="D169" s="145"/>
       <c r="E169" s="112">
         <v>100</v>
       </c>
@@ -9379,11 +9376,11 @@
       <c r="B170" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C170" s="152">
+      <c r="C170" s="145">
         <f>0.95*C169</f>
         <v>456000</v>
       </c>
-      <c r="D170" s="152"/>
+      <c r="D170" s="145"/>
       <c r="E170" s="113">
         <f>C170/C168*100</f>
         <v>86.036937584485301</v>
@@ -9400,11 +9397,11 @@
       <c r="B171" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="C171" s="152">
+      <c r="C171" s="145">
         <f>C168-C170</f>
         <v>74004.917425406631</v>
       </c>
-      <c r="D171" s="152"/>
+      <c r="D171" s="145"/>
       <c r="E171" s="113">
         <f>C171/C169*100</f>
         <v>15.417691130293049</v>
@@ -9421,11 +9418,11 @@
       <c r="B172" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="C172" s="152">
+      <c r="C172" s="145">
         <f>E172*C169/100</f>
         <v>9600</v>
       </c>
-      <c r="D172" s="152"/>
+      <c r="D172" s="145"/>
       <c r="E172" s="113">
         <v>2</v>
       </c>
@@ -9441,11 +9438,11 @@
       <c r="B173" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="C173" s="150">
+      <c r="C173" s="173">
         <f>E173*C169/100</f>
         <v>14400</v>
       </c>
-      <c r="D173" s="150"/>
+      <c r="D173" s="173"/>
       <c r="E173" s="113">
         <v>3</v>
       </c>
@@ -9461,6 +9458,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="C173:D173"/>
+    <mergeCell ref="C167:D167"/>
+    <mergeCell ref="C168:D168"/>
+    <mergeCell ref="C169:D169"/>
+    <mergeCell ref="C170:D170"/>
+    <mergeCell ref="C171:D171"/>
+    <mergeCell ref="C172:D172"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -9468,13 +9472,6 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="C173:D173"/>
-    <mergeCell ref="C167:D167"/>
-    <mergeCell ref="C168:D168"/>
-    <mergeCell ref="C169:D169"/>
-    <mergeCell ref="C170:D170"/>
-    <mergeCell ref="C171:D171"/>
-    <mergeCell ref="C172:D172"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -9504,56 +9501,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="178" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="176" t="s">
+      <c r="B1" s="178" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="176" t="s">
+      <c r="C1" s="178" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="176" t="s">
+      <c r="D1" s="178" t="s">
         <v>163</v>
       </c>
-      <c r="E1" s="176" t="s">
+      <c r="E1" s="178" t="s">
         <v>166</v>
       </c>
-      <c r="F1" s="176" t="s">
+      <c r="F1" s="178" t="s">
         <v>164</v>
       </c>
-      <c r="G1" s="176" t="s">
+      <c r="G1" s="178" t="s">
         <v>165</v>
       </c>
-      <c r="H1" s="176" t="s">
+      <c r="H1" s="178" t="s">
         <v>161</v>
       </c>
-      <c r="I1" s="178" t="s">
+      <c r="I1" s="180" t="s">
         <v>162</v>
       </c>
-      <c r="J1" s="172" t="s">
+      <c r="J1" s="174" t="s">
         <v>167</v>
       </c>
-      <c r="K1" s="175" t="s">
+      <c r="K1" s="177" t="s">
         <v>168</v>
       </c>
-      <c r="L1" s="175"/>
-      <c r="M1" s="173" t="s">
+      <c r="L1" s="177"/>
+      <c r="M1" s="175" t="s">
         <v>169</v>
       </c>
-      <c r="N1" s="173"/>
+      <c r="N1" s="175"/>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="177"/>
-      <c r="B2" s="177"/>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
-      <c r="E2" s="177"/>
-      <c r="F2" s="177"/>
-      <c r="G2" s="177"/>
-      <c r="H2" s="177"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="172"/>
+      <c r="A2" s="179"/>
+      <c r="B2" s="179"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="181"/>
+      <c r="J2" s="174"/>
       <c r="K2" s="127" t="s">
         <v>3</v>
       </c>
@@ -9625,11 +9622,11 @@
         <f>57*J3/1000</f>
         <v>0.45600000000000002</v>
       </c>
-      <c r="M4" s="174">
+      <c r="M4" s="176">
         <f>SQRT(('Size of water tank'!M3)^2+('Size of water tank'!N3)^2)</f>
         <v>0.43103125948585641</v>
       </c>
-      <c r="N4" s="174"/>
+      <c r="N4" s="176"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="FJvrNP3q0MiFodO2bgVO1VomBYM83VDIGAlEPXy+3L7uGnsbugwG4+twkxW5BfXcDD4dyEyGPhARCa/cu3l7XQ==" saltValue="6UJ1dKK5+0v9OnpfIn6j6Q==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
@@ -9655,7 +9652,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD07E67D-5D7A-4E99-87D9-10A521F06797}">
-  <dimension ref="A1:L252"/>
+  <dimension ref="A1:L248"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="4.42578125" style="69" customWidth="1"/>
@@ -9666,101 +9663,101 @@
     <col min="6" max="6" width="8.42578125" style="1" customWidth="1"/>
     <col min="7" max="7" width="10.140625" style="1" customWidth="1"/>
     <col min="8" max="8" width="5.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.7109375" style="1" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="150" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="146"/>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="150"/>
       <c r="L1" s="109"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="147" t="s">
+      <c r="A2" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="147"/>
-      <c r="C2" s="147"/>
-      <c r="D2" s="147"/>
-      <c r="E2" s="147"/>
-      <c r="F2" s="147"/>
-      <c r="G2" s="147"/>
-      <c r="H2" s="147"/>
-      <c r="I2" s="147"/>
-      <c r="J2" s="147"/>
-      <c r="K2" s="147"/>
+      <c r="B2" s="151"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="151"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="151"/>
+      <c r="H2" s="151"/>
+      <c r="I2" s="151"/>
+      <c r="J2" s="151"/>
+      <c r="K2" s="151"/>
       <c r="L2" s="118"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="146" t="s">
+      <c r="A3" s="150" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="146"/>
-      <c r="C3" s="146"/>
-      <c r="D3" s="146"/>
-      <c r="E3" s="146"/>
-      <c r="F3" s="146"/>
-      <c r="G3" s="146"/>
-      <c r="H3" s="146"/>
-      <c r="I3" s="146"/>
-      <c r="J3" s="146"/>
-      <c r="K3" s="146"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="150"/>
+      <c r="D3" s="150"/>
+      <c r="E3" s="150"/>
+      <c r="F3" s="150"/>
+      <c r="G3" s="150"/>
+      <c r="H3" s="150"/>
+      <c r="I3" s="150"/>
+      <c r="J3" s="150"/>
+      <c r="K3" s="150"/>
       <c r="L3" s="109"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="148" t="s">
+      <c r="A4" s="152" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="148"/>
-      <c r="C4" s="148"/>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
-      <c r="F4" s="148"/>
-      <c r="G4" s="148"/>
-      <c r="H4" s="148"/>
-      <c r="I4" s="148"/>
-      <c r="J4" s="148"/>
-      <c r="K4" s="148"/>
+      <c r="B4" s="152"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
+      <c r="F4" s="152"/>
+      <c r="G4" s="152"/>
+      <c r="H4" s="152"/>
+      <c r="I4" s="152"/>
+      <c r="J4" s="152"/>
+      <c r="K4" s="152"/>
     </row>
     <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="119" t="s">
         <v>139</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="J5" s="149" t="s">
+      <c r="J5" s="153" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="149"/>
+      <c r="K5" s="153"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="144" t="s">
+      <c r="A6" s="148" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="144"/>
-      <c r="C6" s="144"/>
-      <c r="D6" s="144"/>
-      <c r="E6" s="144"/>
-      <c r="F6" s="144"/>
+      <c r="B6" s="148"/>
+      <c r="C6" s="148"/>
+      <c r="D6" s="148"/>
+      <c r="E6" s="148"/>
+      <c r="F6" s="148"/>
       <c r="G6" s="61"/>
-      <c r="H6" s="145" t="s">
+      <c r="H6" s="149" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="145"/>
-      <c r="J6" s="145"/>
-      <c r="K6" s="145"/>
+      <c r="I6" s="149"/>
+      <c r="J6" s="149"/>
+      <c r="K6" s="149"/>
     </row>
     <row r="7" spans="1:12">
       <c r="B7" s="3"/>
@@ -11401,7 +11398,7 @@
     <row r="78" spans="1:11">
       <c r="A78" s="134"/>
       <c r="B78" s="142" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C78" s="135">
         <v>1</v>
@@ -11635,11 +11632,11 @@
         <v>1</v>
       </c>
       <c r="D88" s="80">
-        <f>D76</f>
+        <f t="shared" ref="D88:E93" si="9">D76</f>
         <v>3.4034339124250739</v>
       </c>
       <c r="E88" s="80">
-        <f>E76</f>
+        <f t="shared" si="9"/>
         <v>3.2510413491821595</v>
       </c>
       <c r="F88" s="80"/>
@@ -11663,11 +11660,11 @@
         <v>1</v>
       </c>
       <c r="D89" s="80">
-        <f>D77</f>
+        <f t="shared" si="9"/>
         <v>4.1398963730569944</v>
       </c>
       <c r="E89" s="80">
-        <f>E77</f>
+        <f t="shared" si="9"/>
         <v>5.1051508686376099</v>
       </c>
       <c r="F89" s="80"/>
@@ -11691,11 +11688,11 @@
         <v>1</v>
       </c>
       <c r="D90" s="136">
-        <f>D78</f>
+        <f t="shared" si="9"/>
         <v>23.188966778421211</v>
       </c>
       <c r="E90" s="136">
-        <f>E78</f>
+        <f t="shared" si="9"/>
         <v>0.45</v>
       </c>
       <c r="F90" s="136"/>
@@ -11716,11 +11713,11 @@
         <v>1</v>
       </c>
       <c r="D91" s="136">
-        <f>D79</f>
+        <f t="shared" si="9"/>
         <v>6.4004876562023769</v>
       </c>
       <c r="E91" s="136">
-        <f>E79</f>
+        <f t="shared" si="9"/>
         <v>0.9</v>
       </c>
       <c r="F91" s="136"/>
@@ -11741,11 +11738,11 @@
         <v>1</v>
       </c>
       <c r="D92" s="136">
-        <f>D80</f>
+        <f t="shared" si="9"/>
         <v>15.239256324291373</v>
       </c>
       <c r="E92" s="136">
-        <f>E80</f>
+        <f t="shared" si="9"/>
         <v>0.6</v>
       </c>
       <c r="F92" s="136"/>
@@ -11766,11 +11763,11 @@
         <v>1</v>
       </c>
       <c r="D93" s="136">
-        <f>D81</f>
+        <f t="shared" si="9"/>
         <v>10.337397135019812</v>
       </c>
       <c r="E93" s="136">
-        <f>E81</f>
+        <f t="shared" si="9"/>
         <v>0.6</v>
       </c>
       <c r="F93" s="136"/>
@@ -11834,7 +11831,7 @@
       <c r="E96" s="84"/>
       <c r="F96" s="86"/>
       <c r="G96" s="84">
-        <f t="shared" ref="G96" si="9">PRODUCT(C96:F96)</f>
+        <f t="shared" ref="G96" si="10">PRODUCT(C96:F96)</f>
         <v>1</v>
       </c>
       <c r="H96" s="80" t="s">
@@ -11894,7 +11891,7 @@
       <c r="E99" s="80"/>
       <c r="F99" s="80"/>
       <c r="G99" s="84">
-        <f t="shared" ref="G99" si="10">PRODUCT(C99:F99)</f>
+        <f t="shared" ref="G99" si="11">PRODUCT(C99:F99)</f>
         <v>91.600876132689052</v>
       </c>
       <c r="H99" s="80"/>
@@ -11975,7 +11972,7 @@
         <v>0.8</v>
       </c>
       <c r="G103" s="84">
-        <f t="shared" ref="G103" si="11">PRODUCT(C103:F103)</f>
+        <f t="shared" ref="G103" si="12">PRODUCT(C103:F103)</f>
         <v>0.17043584273087475</v>
       </c>
       <c r="H103" s="80"/>
@@ -12054,7 +12051,7 @@
       </c>
       <c r="F107" s="80"/>
       <c r="G107" s="84">
-        <f t="shared" ref="G107:G109" si="12">PRODUCT(C107:F107)</f>
+        <f t="shared" ref="G107:G109" si="13">PRODUCT(C107:F107)</f>
         <v>13.122797927461137</v>
       </c>
       <c r="H107" s="80"/>
@@ -12080,7 +12077,7 @@
       </c>
       <c r="F108" s="136"/>
       <c r="G108" s="84">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-1.0822147892593386</v>
       </c>
       <c r="H108" s="136"/>
@@ -12106,7 +12103,7 @@
       </c>
       <c r="F109" s="136"/>
       <c r="G109" s="84">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1.1611746665872733</v>
       </c>
       <c r="H109" s="136"/>
@@ -12187,7 +12184,7 @@
       </c>
       <c r="F113" s="80"/>
       <c r="G113" s="84">
-        <f t="shared" ref="G113" si="13">PRODUCT(C113:F113)</f>
+        <f t="shared" ref="G113" si="14">PRODUCT(C113:F113)</f>
         <v>1.0822147892593386</v>
       </c>
       <c r="H113" s="80"/>
@@ -12237,7 +12234,7 @@
         <v>17</v>
       </c>
       <c r="B116" s="117" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C116" s="89"/>
       <c r="D116" s="90"/>
@@ -12252,7 +12249,7 @@
     <row r="117" spans="1:11">
       <c r="A117" s="88"/>
       <c r="B117" s="91" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C117" s="89">
         <v>50</v>
@@ -12312,12 +12309,12 @@
       <c r="J119" s="84"/>
       <c r="K119" s="81"/>
     </row>
-    <row r="120" spans="1:11" ht="30.75">
+    <row r="120" spans="1:11" ht="45.75">
       <c r="A120" s="77">
         <v>18</v>
       </c>
       <c r="B120" s="115" t="s">
-        <v>133</v>
+        <v>203</v>
       </c>
       <c r="C120" s="83"/>
       <c r="D120" s="80"/>
@@ -12368,7 +12365,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="G122" s="84">
-        <f t="shared" ref="G122:G153" si="14">PRODUCT(C122:F122)</f>
+        <f t="shared" ref="G122:G153" si="15">PRODUCT(C122:F122)</f>
         <v>4.2240000000000002</v>
       </c>
       <c r="H122" s="80"/>
@@ -12390,7 +12387,7 @@
         <v>1.39</v>
       </c>
       <c r="G123" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>11.12</v>
       </c>
       <c r="H123" s="80"/>
@@ -12413,7 +12410,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="G124" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.2240000000000002</v>
       </c>
       <c r="H124" s="80"/>
@@ -12435,7 +12432,7 @@
         <v>1.3</v>
       </c>
       <c r="G125" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>10.166</v>
       </c>
       <c r="H125" s="80"/>
@@ -12458,7 +12455,7 @@
         <v>2.31</v>
       </c>
       <c r="G126" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.4352</v>
       </c>
       <c r="H126" s="80"/>
@@ -12480,7 +12477,7 @@
         <v>1.37</v>
       </c>
       <c r="G127" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>10.8504</v>
       </c>
       <c r="H127" s="80"/>
@@ -12503,7 +12500,7 @@
         <v>2.29</v>
       </c>
       <c r="G128" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.3967999999999998</v>
       </c>
       <c r="H128" s="80"/>
@@ -12525,7 +12522,7 @@
         <v>1.2649999999999999</v>
       </c>
       <c r="G129" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.8037499999999991</v>
       </c>
       <c r="H129" s="80"/>
@@ -12548,7 +12545,7 @@
         <v>2.19</v>
       </c>
       <c r="G130" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.2047999999999996</v>
       </c>
       <c r="H130" s="80"/>
@@ -12570,7 +12567,7 @@
         <v>1.28</v>
       </c>
       <c r="G131" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.4464000000000006</v>
       </c>
       <c r="H131" s="80"/>
@@ -12593,7 +12590,7 @@
         <v>2.19</v>
       </c>
       <c r="G132" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.2047999999999996</v>
       </c>
       <c r="H132" s="80"/>
@@ -12616,7 +12613,7 @@
         <v>1.1200000000000001</v>
       </c>
       <c r="G133" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.3408000000000015</v>
       </c>
       <c r="H133" s="80"/>
@@ -12639,7 +12636,7 @@
         <v>2.2599999999999998</v>
       </c>
       <c r="G134" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3.0735999999999999</v>
       </c>
       <c r="H134" s="80"/>
@@ -12662,7 +12659,7 @@
         <v>2.15</v>
       </c>
       <c r="G135" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2.9239999999999999</v>
       </c>
       <c r="H135" s="80"/>
@@ -12684,7 +12681,7 @@
         <v>1.1599999999999999</v>
       </c>
       <c r="G136" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>5.8</v>
       </c>
       <c r="H136" s="80"/>
@@ -12707,7 +12704,7 @@
         <v>2.1800000000000002</v>
       </c>
       <c r="G137" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.1856</v>
       </c>
       <c r="H137" s="80"/>
@@ -12729,7 +12726,7 @@
         <v>1.2</v>
       </c>
       <c r="G138" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.4559999999999995</v>
       </c>
       <c r="H138" s="80"/>
@@ -12752,7 +12749,7 @@
         <v>2.15</v>
       </c>
       <c r="G139" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.1280000000000001</v>
       </c>
       <c r="H139" s="80"/>
@@ -12774,7 +12771,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="G140" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.1999999999999993</v>
       </c>
       <c r="H140" s="80"/>
@@ -12797,7 +12794,7 @@
         <v>2.08</v>
       </c>
       <c r="G141" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3.9935999999999998</v>
       </c>
       <c r="H141" s="80"/>
@@ -12819,7 +12816,7 @@
         <v>1.25</v>
       </c>
       <c r="G142" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.9250000000000007</v>
       </c>
       <c r="H142" s="80"/>
@@ -12842,7 +12839,7 @@
         <v>2.25</v>
       </c>
       <c r="G143" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.32</v>
       </c>
       <c r="H143" s="80"/>
@@ -12864,7 +12861,7 @@
         <v>1.23</v>
       </c>
       <c r="G144" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.84</v>
       </c>
       <c r="H144" s="80"/>
@@ -12887,7 +12884,7 @@
         <v>2.25</v>
       </c>
       <c r="G145" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.32</v>
       </c>
       <c r="H145" s="80"/>
@@ -12909,7 +12906,7 @@
         <v>1.32</v>
       </c>
       <c r="G146" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>10.718399999999999</v>
       </c>
       <c r="H146" s="80"/>
@@ -12932,7 +12929,7 @@
         <v>2.1800000000000002</v>
       </c>
       <c r="G147" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.1856</v>
       </c>
       <c r="H147" s="80"/>
@@ -12955,7 +12952,7 @@
         <v>1.32</v>
       </c>
       <c r="G148" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>10.348800000000001</v>
       </c>
       <c r="H148" s="80"/>
@@ -12978,7 +12975,7 @@
         <v>2.2799999999999998</v>
       </c>
       <c r="G149" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.3775999999999993</v>
       </c>
       <c r="H149" s="80"/>
@@ -13000,7 +12997,7 @@
         <v>1.32</v>
       </c>
       <c r="G150" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>9.5568000000000008</v>
       </c>
       <c r="H150" s="80"/>
@@ -13023,7 +13020,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="G151" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4.2240000000000002</v>
       </c>
       <c r="H151" s="80"/>
@@ -13046,7 +13043,7 @@
         <v>1.35</v>
       </c>
       <c r="G152" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>-9.9360000000000017</v>
       </c>
       <c r="H152" s="80"/>
@@ -13057,7 +13054,7 @@
     <row r="153" spans="1:11">
       <c r="A153" s="134"/>
       <c r="B153" s="142" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C153" s="135">
         <v>1</v>
@@ -13072,7 +13069,7 @@
         <v>0.52</v>
       </c>
       <c r="G153" s="84">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>10.24880219445291</v>
       </c>
       <c r="H153" s="136"/>
@@ -13096,7 +13093,7 @@
         <v>0.52</v>
       </c>
       <c r="G154" s="84">
-        <f t="shared" ref="G154:G155" si="15">PRODUCT(C154:F154)</f>
+        <f t="shared" ref="G154" si="16">PRODUCT(C154:F154)</f>
         <v>9.6148491313623889</v>
       </c>
       <c r="H154" s="136"/>
@@ -13106,79 +13103,89 @@
     </row>
     <row r="155" spans="1:11">
       <c r="A155" s="134"/>
-      <c r="B155" s="142" t="s">
-        <v>186</v>
-      </c>
-      <c r="C155" s="135">
-        <v>2</v>
-      </c>
-      <c r="D155" s="136">
-        <f>2.5/3.281</f>
-        <v>0.76196281621456874</v>
-      </c>
+      <c r="B155" s="120" t="s">
+        <v>189</v>
+      </c>
+      <c r="C155" s="135"/>
+      <c r="D155" s="136"/>
       <c r="E155" s="136"/>
-      <c r="F155" s="136">
-        <f>7/3.281</f>
-        <v>2.1334958854007922</v>
-      </c>
-      <c r="G155" s="139">
-        <f t="shared" si="15"/>
-        <v>3.251289066444365</v>
-      </c>
+      <c r="F155" s="136"/>
+      <c r="G155" s="136"/>
       <c r="H155" s="136"/>
       <c r="I155" s="136"/>
       <c r="J155" s="136"/>
       <c r="K155" s="137"/>
     </row>
     <row r="156" spans="1:11">
-      <c r="A156" s="77"/>
-      <c r="B156" s="92"/>
-      <c r="C156" s="83"/>
-      <c r="D156" s="80"/>
-      <c r="E156" s="80"/>
-      <c r="F156" s="80"/>
-      <c r="G156" s="80">
-        <f>SUM(G121:G155)</f>
-        <v>223.93979039225965</v>
-      </c>
-      <c r="H156" s="80" t="s">
-        <v>23</v>
-      </c>
-      <c r="I156" s="80">
-        <f>1.15*253.8</f>
-        <v>291.87</v>
-      </c>
-      <c r="J156" s="80">
-        <f>G156*I156</f>
-        <v>65361.306621788826</v>
-      </c>
-      <c r="K156" s="81"/>
+      <c r="A156" s="134"/>
+      <c r="B156" s="142" t="s">
+        <v>197</v>
+      </c>
+      <c r="C156" s="135">
+        <v>1</v>
+      </c>
+      <c r="D156" s="136">
+        <f>2*(29.917/3.281)+2*(28.5/3.281)</f>
+        <v>35.609265467845169</v>
+      </c>
+      <c r="E156" s="136"/>
+      <c r="F156" s="136">
+        <f>9.33/3.281</f>
+        <v>2.8436452301127706</v>
+      </c>
+      <c r="G156" s="84">
+        <f t="shared" ref="G156:G161" si="17">PRODUCT(C156:F156)</f>
+        <v>101.26011789545731</v>
+      </c>
+      <c r="H156" s="136"/>
+      <c r="I156" s="136"/>
+      <c r="J156" s="136"/>
+      <c r="K156" s="137"/>
     </row>
     <row r="157" spans="1:11">
-      <c r="A157" s="77"/>
-      <c r="B157" s="92"/>
-      <c r="C157" s="83"/>
-      <c r="D157" s="80"/>
-      <c r="E157" s="80"/>
-      <c r="F157" s="80"/>
-      <c r="G157" s="80"/>
-      <c r="H157" s="80"/>
-      <c r="I157" s="80"/>
-      <c r="J157" s="80"/>
-      <c r="K157" s="81"/>
-    </row>
-    <row r="158" spans="1:11" ht="30.75">
-      <c r="A158" s="134">
-        <v>19</v>
-      </c>
-      <c r="B158" s="115" t="s">
-        <v>184</v>
-      </c>
-      <c r="C158" s="135"/>
-      <c r="D158" s="136"/>
+      <c r="A157" s="134"/>
+      <c r="B157" s="142" t="s">
+        <v>187</v>
+      </c>
+      <c r="C157" s="135">
+        <v>-1</v>
+      </c>
+      <c r="D157" s="136">
+        <v>1.2</v>
+      </c>
+      <c r="E157" s="136"/>
+      <c r="F157" s="136">
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="G157" s="84">
+        <f t="shared" si="17"/>
+        <v>-2.9259372142639433</v>
+      </c>
+      <c r="H157" s="136"/>
+      <c r="I157" s="136"/>
+      <c r="J157" s="136"/>
+      <c r="K157" s="137"/>
+    </row>
+    <row r="158" spans="1:11">
+      <c r="A158" s="134"/>
+      <c r="B158" s="142" t="s">
+        <v>188</v>
+      </c>
+      <c r="C158" s="135">
+        <v>-1</v>
+      </c>
+      <c r="D158" s="136">
+        <v>0.9</v>
+      </c>
       <c r="E158" s="136"/>
-      <c r="F158" s="136"/>
-      <c r="G158" s="136"/>
+      <c r="F158" s="136">
+        <v>1.8</v>
+      </c>
+      <c r="G158" s="84">
+        <f t="shared" si="17"/>
+        <v>-1.62</v>
+      </c>
       <c r="H158" s="136"/>
       <c r="I158" s="136"/>
       <c r="J158" s="136"/>
@@ -13186,24 +13193,20 @@
     </row>
     <row r="159" spans="1:11">
       <c r="A159" s="134"/>
-      <c r="B159" s="142" t="s">
-        <v>185</v>
-      </c>
+      <c r="B159" s="142"/>
       <c r="C159" s="135">
-        <v>1</v>
+        <v>-6</v>
       </c>
       <c r="D159" s="136">
-        <f>(2*(12.33+13))/3.281</f>
-        <v>15.440414507772019</v>
+        <v>1.8</v>
       </c>
       <c r="E159" s="136"/>
       <c r="F159" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
+        <v>1.2</v>
       </c>
       <c r="G159" s="84">
-        <f t="shared" ref="G159:G162" si="16">PRODUCT(C159:F159)</f>
-        <v>41.177576026517876</v>
+        <f t="shared" si="17"/>
+        <v>-12.96</v>
       </c>
       <c r="H159" s="136"/>
       <c r="I159" s="136"/>
@@ -13212,24 +13215,20 @@
     </row>
     <row r="160" spans="1:11">
       <c r="A160" s="134"/>
-      <c r="B160" s="142" t="s">
-        <v>187</v>
-      </c>
+      <c r="B160" s="142"/>
       <c r="C160" s="135">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D160" s="136">
-        <f>12.33/3.281</f>
-        <v>3.7580006095702529</v>
-      </c>
-      <c r="E160" s="136">
-        <f>13/3.281</f>
-        <v>3.9622066443157573</v>
-      </c>
-      <c r="F160" s="136"/>
+        <v>1.2</v>
+      </c>
+      <c r="E160" s="136"/>
+      <c r="F160" s="136">
+        <v>1.2</v>
+      </c>
       <c r="G160" s="84">
-        <f t="shared" si="16"/>
-        <v>14.889974984581922</v>
+        <f t="shared" si="17"/>
+        <v>-1.44</v>
       </c>
       <c r="H160" s="136"/>
       <c r="I160" s="136"/>
@@ -13238,24 +13237,20 @@
     </row>
     <row r="161" spans="1:11">
       <c r="A161" s="134"/>
-      <c r="B161" s="142" t="s">
-        <v>188</v>
-      </c>
+      <c r="B161" s="142"/>
       <c r="C161" s="135">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D161" s="136">
-        <f>(2*(17.25+13.42))/3.281</f>
-        <v>18.695519658640659</v>
+        <v>0.9</v>
       </c>
       <c r="E161" s="136"/>
       <c r="F161" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
-      </c>
-      <c r="G161" s="84">
-        <f t="shared" si="16"/>
-        <v>49.858517833924338</v>
+        <v>1.2</v>
+      </c>
+      <c r="G161" s="139">
+        <f t="shared" si="17"/>
+        <v>-1.08</v>
       </c>
       <c r="H161" s="136"/>
       <c r="I161" s="136"/>
@@ -13264,25 +13259,14 @@
     </row>
     <row r="162" spans="1:11">
       <c r="A162" s="134"/>
-      <c r="B162" s="142" t="s">
-        <v>187</v>
-      </c>
-      <c r="C162" s="135">
-        <v>1</v>
-      </c>
-      <c r="D162" s="136">
-        <f>17.25/3.281</f>
-        <v>5.2575434318805243</v>
-      </c>
-      <c r="E162" s="136">
-        <f>13.42/3.281</f>
-        <v>4.0902163974398045</v>
-      </c>
+      <c r="B162" s="120" t="s">
+        <v>192</v>
+      </c>
+      <c r="C162" s="135"/>
+      <c r="D162" s="136"/>
+      <c r="E162" s="136"/>
       <c r="F162" s="136"/>
-      <c r="G162" s="84">
-        <f t="shared" si="16"/>
-        <v>21.504490355329665</v>
-      </c>
+      <c r="G162" s="84"/>
       <c r="H162" s="136"/>
       <c r="I162" s="136"/>
       <c r="J162" s="136"/>
@@ -13291,23 +13275,23 @@
     <row r="163" spans="1:11">
       <c r="A163" s="134"/>
       <c r="B163" s="142" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C163" s="135">
         <v>1</v>
       </c>
       <c r="D163" s="136">
-        <f>(2*(10.833+13.42))/3.281</f>
-        <v>14.783907345321548</v>
+        <f>2*(29.917/3.281)+2*(28.5/3.281)</f>
+        <v>35.609265467845169</v>
       </c>
       <c r="E163" s="136"/>
       <c r="F163" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
+        <f>9.33/3.281</f>
+        <v>2.8436452301127706</v>
       </c>
       <c r="G163" s="84">
-        <f t="shared" ref="G163:G167" si="17">PRODUCT(C163:F163)</f>
-        <v>39.426756864237589</v>
+        <f t="shared" ref="G163:G168" si="18">PRODUCT(C163:F163)</f>
+        <v>101.26011789545731</v>
       </c>
       <c r="H163" s="136"/>
       <c r="I163" s="136"/>
@@ -13320,20 +13304,19 @@
         <v>187</v>
       </c>
       <c r="C164" s="135">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D164" s="136">
-        <f>10.833/3.281</f>
-        <v>3.3017372752209693</v>
-      </c>
-      <c r="E164" s="136">
-        <f>13.42/3.281</f>
-        <v>4.0902163974398045</v>
-      </c>
-      <c r="F164" s="136"/>
+        <f>3.5/3.281</f>
+        <v>1.0667479427003961</v>
+      </c>
+      <c r="E164" s="136"/>
+      <c r="F164" s="136">
+        <v>2.1</v>
+      </c>
       <c r="G164" s="84">
-        <f t="shared" si="17"/>
-        <v>13.504819943147028</v>
+        <f t="shared" si="18"/>
+        <v>-2.2401706796708321</v>
       </c>
       <c r="H164" s="136"/>
       <c r="I164" s="136"/>
@@ -13343,23 +13326,21 @@
     <row r="165" spans="1:11">
       <c r="A165" s="134"/>
       <c r="B165" s="142" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C165" s="135">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="D165" s="136">
-        <f>3.5/3.281</f>
-        <v>1.0667479427003961</v>
+        <v>0.9</v>
       </c>
       <c r="E165" s="136"/>
       <c r="F165" s="136">
-        <f>7/3.281</f>
-        <v>2.1334958854007922</v>
+        <v>1.8</v>
       </c>
       <c r="G165" s="84">
-        <f t="shared" si="17"/>
-        <v>-6.8277070395331645</v>
+        <f t="shared" si="18"/>
+        <v>-1.62</v>
       </c>
       <c r="H165" s="136"/>
       <c r="I165" s="136"/>
@@ -13368,24 +13349,20 @@
     </row>
     <row r="166" spans="1:11">
       <c r="A166" s="134"/>
-      <c r="B166" s="142" t="s">
-        <v>192</v>
-      </c>
+      <c r="B166" s="142"/>
       <c r="C166" s="135">
         <v>-6</v>
       </c>
       <c r="D166" s="136">
-        <f>6/3.281</f>
-        <v>1.8287107589149649</v>
+        <v>1.8</v>
       </c>
       <c r="E166" s="136"/>
       <c r="F166" s="136">
-        <f>4/3.281</f>
-        <v>1.2191405059433098</v>
+        <v>1.2</v>
       </c>
       <c r="G166" s="84">
-        <f t="shared" si="17"/>
-        <v>-13.376732159085387</v>
+        <f t="shared" si="18"/>
+        <v>-12.96</v>
       </c>
       <c r="H166" s="136"/>
       <c r="I166" s="136"/>
@@ -13399,17 +13376,15 @@
         <v>-1</v>
       </c>
       <c r="D167" s="136">
-        <f>4/3.281</f>
-        <v>1.2191405059433098</v>
+        <v>1.2</v>
       </c>
       <c r="E167" s="136"/>
       <c r="F167" s="136">
-        <f>4/3.281</f>
-        <v>1.2191405059433098</v>
+        <v>1.2</v>
       </c>
       <c r="G167" s="84">
-        <f t="shared" si="17"/>
-        <v>-1.4863035732317094</v>
+        <f t="shared" si="18"/>
+        <v>-1.44</v>
       </c>
       <c r="H167" s="136"/>
       <c r="I167" s="136"/>
@@ -13417,132 +13392,117 @@
       <c r="K167" s="137"/>
     </row>
     <row r="168" spans="1:11">
-      <c r="A168" s="77"/>
-      <c r="B168" s="92"/>
-      <c r="C168" s="83"/>
-      <c r="D168" s="80"/>
-      <c r="E168" s="80"/>
-      <c r="F168" s="80"/>
-      <c r="G168" s="80">
-        <f>SUM(G159:G167)</f>
-        <v>158.67139323588816</v>
-      </c>
-      <c r="H168" s="80" t="s">
-        <v>23</v>
-      </c>
-      <c r="I168" s="80">
-        <f>1.15*300.03</f>
-        <v>345.03449999999992</v>
-      </c>
-      <c r="J168" s="80">
-        <f>G168*I168</f>
-        <v>54747.104829448042</v>
-      </c>
-      <c r="K168" s="81"/>
+      <c r="A168" s="134"/>
+      <c r="B168" s="142"/>
+      <c r="C168" s="135">
+        <v>-1</v>
+      </c>
+      <c r="D168" s="136">
+        <v>0.9</v>
+      </c>
+      <c r="E168" s="136"/>
+      <c r="F168" s="136">
+        <v>1.2</v>
+      </c>
+      <c r="G168" s="139">
+        <f t="shared" si="18"/>
+        <v>-1.08</v>
+      </c>
+      <c r="H168" s="136"/>
+      <c r="I168" s="136"/>
+      <c r="J168" s="136"/>
+      <c r="K168" s="137"/>
     </row>
     <row r="169" spans="1:11">
       <c r="A169" s="134"/>
-      <c r="B169" s="133"/>
+      <c r="B169" s="143" t="s">
+        <v>194</v>
+      </c>
       <c r="C169" s="135"/>
       <c r="D169" s="136"/>
       <c r="E169" s="136"/>
       <c r="F169" s="136"/>
-      <c r="G169" s="136"/>
+      <c r="G169" s="84"/>
       <c r="H169" s="136"/>
       <c r="I169" s="136"/>
       <c r="J169" s="136"/>
       <c r="K169" s="137"/>
     </row>
-    <row r="170" spans="1:11" ht="30.75">
-      <c r="A170" s="134">
-        <v>20</v>
-      </c>
-      <c r="B170" s="115" t="s">
-        <v>190</v>
-      </c>
-      <c r="C170" s="135"/>
-      <c r="D170" s="136"/>
+    <row r="170" spans="1:11">
+      <c r="A170" s="134"/>
+      <c r="B170" s="142" t="s">
+        <v>198</v>
+      </c>
+      <c r="C170" s="135">
+        <v>1</v>
+      </c>
+      <c r="D170" s="136">
+        <f>(11.833/3.281)+(14.833/3.281)</f>
+        <v>8.1274001828710745</v>
+      </c>
       <c r="E170" s="136"/>
-      <c r="F170" s="136"/>
-      <c r="G170" s="136"/>
+      <c r="F170" s="136">
+        <f>9.33/3.281</f>
+        <v>2.8436452301127706</v>
+      </c>
+      <c r="G170" s="84">
+        <f t="shared" ref="G170" si="19">PRODUCT(C170:F170)</f>
+        <v>23.11144276323899</v>
+      </c>
       <c r="H170" s="136"/>
       <c r="I170" s="136"/>
       <c r="J170" s="136"/>
       <c r="K170" s="137"/>
     </row>
     <row r="171" spans="1:11">
-      <c r="A171" s="134"/>
-      <c r="B171" s="142" t="s">
-        <v>188</v>
-      </c>
-      <c r="C171" s="135">
-        <v>1</v>
-      </c>
-      <c r="D171" s="136">
-        <f>17.25/3.281</f>
-        <v>5.2575434318805243</v>
-      </c>
-      <c r="E171" s="136"/>
-      <c r="F171" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
-      </c>
-      <c r="G171" s="84">
-        <f t="shared" ref="G171:G175" si="18">PRODUCT(C171:F171)</f>
-        <v>14.021184099041324</v>
-      </c>
-      <c r="H171" s="136"/>
-      <c r="I171" s="136"/>
-      <c r="J171" s="136"/>
-      <c r="K171" s="137"/>
+      <c r="A171" s="77"/>
+      <c r="B171" s="92"/>
+      <c r="C171" s="83"/>
+      <c r="D171" s="80"/>
+      <c r="E171" s="80"/>
+      <c r="F171" s="80"/>
+      <c r="G171" s="80">
+        <f>SUM(G121:G170)</f>
+        <v>406.95407198603414</v>
+      </c>
+      <c r="H171" s="80" t="s">
+        <v>23</v>
+      </c>
+      <c r="I171" s="80">
+        <f>1.15*253.8</f>
+        <v>291.87</v>
+      </c>
+      <c r="J171" s="80">
+        <f>G171*I171</f>
+        <v>118777.68499056378</v>
+      </c>
+      <c r="K171" s="81"/>
     </row>
     <row r="172" spans="1:11">
-      <c r="A172" s="134"/>
-      <c r="B172" s="142" t="s">
-        <v>189</v>
-      </c>
-      <c r="C172" s="135">
-        <v>1</v>
-      </c>
-      <c r="D172" s="136">
-        <f>(2*(10.833))/3.281</f>
-        <v>6.6034745504419385</v>
-      </c>
-      <c r="E172" s="136"/>
-      <c r="F172" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
-      </c>
-      <c r="G172" s="84">
-        <f t="shared" si="18"/>
-        <v>17.610607228395903</v>
-      </c>
-      <c r="H172" s="136"/>
-      <c r="I172" s="136"/>
-      <c r="J172" s="136"/>
-      <c r="K172" s="137"/>
-    </row>
-    <row r="173" spans="1:11">
-      <c r="A173" s="134"/>
-      <c r="B173" s="142" t="s">
-        <v>191</v>
-      </c>
-      <c r="C173" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D173" s="136">
-        <f>3.5/3.281</f>
-        <v>1.0667479427003961</v>
-      </c>
+      <c r="A172" s="77"/>
+      <c r="B172" s="92"/>
+      <c r="C172" s="83"/>
+      <c r="D172" s="80"/>
+      <c r="E172" s="80"/>
+      <c r="F172" s="80"/>
+      <c r="G172" s="80"/>
+      <c r="H172" s="80"/>
+      <c r="I172" s="80"/>
+      <c r="J172" s="80"/>
+      <c r="K172" s="81"/>
+    </row>
+    <row r="173" spans="1:11" ht="45.75">
+      <c r="A173" s="134">
+        <v>19</v>
+      </c>
+      <c r="B173" s="115" t="s">
+        <v>204</v>
+      </c>
+      <c r="C173" s="135"/>
+      <c r="D173" s="136"/>
       <c r="E173" s="136"/>
-      <c r="F173" s="136">
-        <f>7/3.281</f>
-        <v>2.1334958854007922</v>
-      </c>
-      <c r="G173" s="84">
-        <f t="shared" si="18"/>
-        <v>-2.2759023465110548</v>
-      </c>
+      <c r="F173" s="136"/>
+      <c r="G173" s="136"/>
       <c r="H173" s="136"/>
       <c r="I173" s="136"/>
       <c r="J173" s="136"/>
@@ -13551,23 +13511,23 @@
     <row r="174" spans="1:11">
       <c r="A174" s="134"/>
       <c r="B174" s="142" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="C174" s="135">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="D174" s="136">
-        <f>6/3.281</f>
-        <v>1.8287107589149649</v>
+        <f>(2*(12.33+13))/3.281</f>
+        <v>15.440414507772019</v>
       </c>
       <c r="E174" s="136"/>
       <c r="F174" s="136">
-        <f>4/3.281</f>
-        <v>1.2191405059433098</v>
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
       </c>
       <c r="G174" s="84">
-        <f t="shared" si="18"/>
-        <v>-4.4589107196951288</v>
+        <f t="shared" ref="G174:G177" si="20">PRODUCT(C174:F174)</f>
+        <v>41.177576026517876</v>
       </c>
       <c r="H174" s="136"/>
       <c r="I174" s="136"/>
@@ -13576,22 +13536,24 @@
     </row>
     <row r="175" spans="1:11">
       <c r="A175" s="134"/>
-      <c r="B175" s="142"/>
+      <c r="B175" s="142" t="s">
+        <v>184</v>
+      </c>
       <c r="C175" s="135">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D175" s="136">
-        <f>4/3.281</f>
-        <v>1.2191405059433098</v>
-      </c>
-      <c r="E175" s="136"/>
-      <c r="F175" s="136">
-        <f>4/3.281</f>
-        <v>1.2191405059433098</v>
-      </c>
+        <f>12.33/3.281</f>
+        <v>3.7580006095702529</v>
+      </c>
+      <c r="E175" s="136">
+        <f>13/3.281</f>
+        <v>3.9622066443157573</v>
+      </c>
+      <c r="F175" s="136"/>
       <c r="G175" s="84">
-        <f t="shared" si="18"/>
-        <v>-1.4863035732317094</v>
+        <f t="shared" si="20"/>
+        <v>14.889974984581922</v>
       </c>
       <c r="H175" s="136"/>
       <c r="I175" s="136"/>
@@ -13599,54 +13561,78 @@
       <c r="K175" s="137"/>
     </row>
     <row r="176" spans="1:11">
-      <c r="A176" s="77"/>
-      <c r="B176" s="92"/>
-      <c r="C176" s="83"/>
-      <c r="D176" s="80"/>
-      <c r="E176" s="80"/>
-      <c r="F176" s="80"/>
-      <c r="G176" s="80">
-        <f>SUM(G171:G175)</f>
-        <v>23.410674687999336</v>
-      </c>
-      <c r="H176" s="80" t="s">
-        <v>23</v>
-      </c>
-      <c r="I176" s="80">
-        <f>1.15*60.3</f>
-        <v>69.344999999999985</v>
-      </c>
-      <c r="J176" s="80">
-        <f>G176*I176</f>
-        <v>1623.4132362393136</v>
-      </c>
-      <c r="K176" s="81"/>
+      <c r="A176" s="134"/>
+      <c r="B176" s="142" t="s">
+        <v>185</v>
+      </c>
+      <c r="C176" s="135">
+        <v>1</v>
+      </c>
+      <c r="D176" s="136">
+        <f>(2*(17.25+13.42))/3.281</f>
+        <v>18.695519658640659</v>
+      </c>
+      <c r="E176" s="136"/>
+      <c r="F176" s="136">
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
+      </c>
+      <c r="G176" s="84">
+        <f t="shared" si="20"/>
+        <v>49.858517833924338</v>
+      </c>
+      <c r="H176" s="136"/>
+      <c r="I176" s="136"/>
+      <c r="J176" s="136"/>
+      <c r="K176" s="137"/>
     </row>
     <row r="177" spans="1:11">
       <c r="A177" s="134"/>
-      <c r="B177" s="133"/>
-      <c r="C177" s="135"/>
-      <c r="D177" s="136"/>
-      <c r="E177" s="136"/>
+      <c r="B177" s="142" t="s">
+        <v>184</v>
+      </c>
+      <c r="C177" s="135">
+        <v>1</v>
+      </c>
+      <c r="D177" s="136">
+        <f>17.25/3.281</f>
+        <v>5.2575434318805243</v>
+      </c>
+      <c r="E177" s="136">
+        <f>13.42/3.281</f>
+        <v>4.0902163974398045</v>
+      </c>
       <c r="F177" s="136"/>
-      <c r="G177" s="136"/>
+      <c r="G177" s="84">
+        <f t="shared" si="20"/>
+        <v>21.504490355329665</v>
+      </c>
       <c r="H177" s="136"/>
       <c r="I177" s="136"/>
       <c r="J177" s="136"/>
       <c r="K177" s="137"/>
     </row>
-    <row r="178" spans="1:11" ht="30.75">
-      <c r="A178" s="134">
-        <v>21</v>
-      </c>
-      <c r="B178" s="115" t="s">
-        <v>193</v>
-      </c>
-      <c r="C178" s="135"/>
-      <c r="D178" s="136"/>
+    <row r="178" spans="1:11">
+      <c r="A178" s="134"/>
+      <c r="B178" s="142" t="s">
+        <v>186</v>
+      </c>
+      <c r="C178" s="135">
+        <v>1</v>
+      </c>
+      <c r="D178" s="136">
+        <f>(2*(10.833+13.42))/3.281</f>
+        <v>14.783907345321548</v>
+      </c>
       <c r="E178" s="136"/>
-      <c r="F178" s="136"/>
-      <c r="G178" s="136"/>
+      <c r="F178" s="136">
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
+      </c>
+      <c r="G178" s="84">
+        <f t="shared" ref="G178:G182" si="21">PRODUCT(C178:F178)</f>
+        <v>39.426756864237589</v>
+      </c>
       <c r="H178" s="136"/>
       <c r="I178" s="136"/>
       <c r="J178" s="136"/>
@@ -13654,14 +13640,25 @@
     </row>
     <row r="179" spans="1:11">
       <c r="A179" s="134"/>
-      <c r="B179" s="120" t="s">
-        <v>194</v>
-      </c>
-      <c r="C179" s="135"/>
-      <c r="D179" s="136"/>
-      <c r="E179" s="136"/>
+      <c r="B179" s="142" t="s">
+        <v>184</v>
+      </c>
+      <c r="C179" s="135">
+        <v>1</v>
+      </c>
+      <c r="D179" s="136">
+        <f>10.833/3.281</f>
+        <v>3.3017372752209693</v>
+      </c>
+      <c r="E179" s="136">
+        <f>13.42/3.281</f>
+        <v>4.0902163974398045</v>
+      </c>
       <c r="F179" s="136"/>
-      <c r="G179" s="136"/>
+      <c r="G179" s="84">
+        <f t="shared" si="21"/>
+        <v>13.504819943147028</v>
+      </c>
       <c r="H179" s="136"/>
       <c r="I179" s="136"/>
       <c r="J179" s="136"/>
@@ -13670,49 +13667,49 @@
     <row r="180" spans="1:11">
       <c r="A180" s="134"/>
       <c r="B180" s="142" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C180" s="135">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="D180" s="136">
-        <f>2*(28.25/3.281)+2*(13.42/3.281)</f>
-        <v>25.400792441328861</v>
+        <f>3.5/3.281</f>
+        <v>1.0667479427003961</v>
       </c>
       <c r="E180" s="136"/>
       <c r="F180" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
+        <f>7/3.281</f>
+        <v>2.1334958854007922</v>
       </c>
       <c r="G180" s="84">
-        <f t="shared" ref="G180:G187" si="19">PRODUCT(C180:F180)</f>
-        <v>67.74060769936834</v>
+        <f t="shared" si="21"/>
+        <v>-6.8277070395331645</v>
       </c>
       <c r="H180" s="136"/>
       <c r="I180" s="136"/>
       <c r="J180" s="136"/>
       <c r="K180" s="137"/>
     </row>
-    <row r="181" spans="1:11" ht="31.5">
+    <row r="181" spans="1:11">
       <c r="A181" s="134"/>
       <c r="B181" s="142" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="C181" s="135">
-        <v>1</v>
+        <v>-6</v>
       </c>
       <c r="D181" s="136">
-        <f>2*(28.25/3.281)+2*(13.083/3.281)</f>
-        <v>25.195367266077415</v>
+        <f>6/3.281</f>
+        <v>1.8287107589149649</v>
       </c>
       <c r="E181" s="136"/>
       <c r="F181" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
+        <f>4/3.281</f>
+        <v>1.2191405059433098</v>
       </c>
       <c r="G181" s="84">
-        <f t="shared" si="19"/>
-        <v>67.192765491672461</v>
+        <f t="shared" si="21"/>
+        <v>-13.376732159085387</v>
       </c>
       <c r="H181" s="136"/>
       <c r="I181" s="136"/>
@@ -13721,23 +13718,22 @@
     </row>
     <row r="182" spans="1:11">
       <c r="A182" s="134"/>
-      <c r="B182" s="142" t="s">
-        <v>191</v>
-      </c>
+      <c r="B182" s="142"/>
       <c r="C182" s="135">
         <v>-1</v>
       </c>
       <c r="D182" s="136">
-        <v>1.2</v>
+        <f>4/3.281</f>
+        <v>1.2191405059433098</v>
       </c>
       <c r="E182" s="136"/>
       <c r="F182" s="136">
-        <f>8/3.281</f>
-        <v>2.4382810118866196</v>
+        <f>4/3.281</f>
+        <v>1.2191405059433098</v>
       </c>
       <c r="G182" s="84">
-        <f t="shared" si="19"/>
-        <v>-2.9259372142639433</v>
+        <f t="shared" si="21"/>
+        <v>-1.4863035732317094</v>
       </c>
       <c r="H182" s="136"/>
       <c r="I182" s="136"/>
@@ -13745,69 +13741,54 @@
       <c r="K182" s="137"/>
     </row>
     <row r="183" spans="1:11">
-      <c r="A183" s="134"/>
-      <c r="B183" s="142"/>
-      <c r="C183" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D183" s="136">
-        <f t="shared" ref="D183" si="20">3.5/3.281</f>
-        <v>1.0667479427003961</v>
-      </c>
-      <c r="E183" s="136"/>
-      <c r="F183" s="136">
-        <v>2.1</v>
-      </c>
-      <c r="G183" s="84">
-        <f t="shared" ref="G183:G184" si="21">PRODUCT(C183:F183)</f>
-        <v>-2.2401706796708321</v>
-      </c>
-      <c r="H183" s="136"/>
-      <c r="I183" s="136"/>
-      <c r="J183" s="136"/>
-      <c r="K183" s="137"/>
+      <c r="A183" s="77"/>
+      <c r="B183" s="92"/>
+      <c r="C183" s="83"/>
+      <c r="D183" s="80"/>
+      <c r="E183" s="80"/>
+      <c r="F183" s="80"/>
+      <c r="G183" s="80">
+        <f>SUM(G174:G182)</f>
+        <v>158.67139323588816</v>
+      </c>
+      <c r="H183" s="80" t="s">
+        <v>23</v>
+      </c>
+      <c r="I183" s="80">
+        <f>1.15*300.03</f>
+        <v>345.03449999999992</v>
+      </c>
+      <c r="J183" s="80">
+        <f>G183*I183</f>
+        <v>54747.104829448042</v>
+      </c>
+      <c r="K183" s="81"/>
     </row>
     <row r="184" spans="1:11">
       <c r="A184" s="134"/>
-      <c r="B184" s="142"/>
-      <c r="C184" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D184" s="136">
-        <v>0.75</v>
-      </c>
+      <c r="B184" s="133"/>
+      <c r="C184" s="135"/>
+      <c r="D184" s="136"/>
       <c r="E184" s="136"/>
-      <c r="F184" s="136">
-        <v>1.8</v>
-      </c>
-      <c r="G184" s="84">
-        <f t="shared" si="21"/>
-        <v>-1.35</v>
-      </c>
+      <c r="F184" s="136"/>
+      <c r="G184" s="136"/>
       <c r="H184" s="136"/>
       <c r="I184" s="136"/>
       <c r="J184" s="136"/>
       <c r="K184" s="137"/>
     </row>
-    <row r="185" spans="1:11">
-      <c r="A185" s="134"/>
-      <c r="B185" s="142" t="s">
-        <v>192</v>
-      </c>
-      <c r="C185" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D185" s="136">
-        <v>0.9</v>
-      </c>
+    <row r="185" spans="1:11" ht="30.75">
+      <c r="A185" s="134">
+        <v>20</v>
+      </c>
+      <c r="B185" s="115" t="s">
+        <v>205</v>
+      </c>
+      <c r="C185" s="135"/>
+      <c r="D185" s="136"/>
       <c r="E185" s="136"/>
-      <c r="F185" s="136">
-        <v>1.8</v>
-      </c>
-      <c r="G185" s="84">
-        <f t="shared" si="19"/>
-        <v>-1.62</v>
-      </c>
+      <c r="F185" s="136"/>
+      <c r="G185" s="136"/>
       <c r="H185" s="136"/>
       <c r="I185" s="136"/>
       <c r="J185" s="136"/>
@@ -13815,20 +13796,24 @@
     </row>
     <row r="186" spans="1:11">
       <c r="A186" s="134"/>
-      <c r="B186" s="142"/>
+      <c r="B186" s="142" t="s">
+        <v>185</v>
+      </c>
       <c r="C186" s="135">
-        <v>-6</v>
+        <v>1</v>
       </c>
       <c r="D186" s="136">
-        <v>1.8</v>
+        <f>17.25/3.281</f>
+        <v>5.2575434318805243</v>
       </c>
       <c r="E186" s="136"/>
       <c r="F186" s="136">
-        <v>1.2</v>
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
       </c>
       <c r="G186" s="84">
-        <f t="shared" si="19"/>
-        <v>-12.96</v>
+        <f t="shared" ref="G186:G190" si="22">PRODUCT(C186:F186)</f>
+        <v>14.021184099041324</v>
       </c>
       <c r="H186" s="136"/>
       <c r="I186" s="136"/>
@@ -13837,20 +13822,24 @@
     </row>
     <row r="187" spans="1:11">
       <c r="A187" s="134"/>
-      <c r="B187" s="142"/>
+      <c r="B187" s="142" t="s">
+        <v>186</v>
+      </c>
       <c r="C187" s="135">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D187" s="136">
-        <v>1.2</v>
+        <f>(2*(10.833))/3.281</f>
+        <v>6.6034745504419385</v>
       </c>
       <c r="E187" s="136"/>
       <c r="F187" s="136">
-        <v>1.2</v>
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
       </c>
       <c r="G187" s="84">
-        <f t="shared" si="19"/>
-        <v>-1.44</v>
+        <f t="shared" si="22"/>
+        <v>17.610607228395903</v>
       </c>
       <c r="H187" s="136"/>
       <c r="I187" s="136"/>
@@ -13859,14 +13848,25 @@
     </row>
     <row r="188" spans="1:11">
       <c r="A188" s="134"/>
-      <c r="B188" s="120" t="s">
-        <v>197</v>
-      </c>
-      <c r="C188" s="135"/>
-      <c r="D188" s="136"/>
+      <c r="B188" s="142" t="s">
+        <v>187</v>
+      </c>
+      <c r="C188" s="135">
+        <v>-1</v>
+      </c>
+      <c r="D188" s="136">
+        <f>3.5/3.281</f>
+        <v>1.0667479427003961</v>
+      </c>
       <c r="E188" s="136"/>
-      <c r="F188" s="136"/>
-      <c r="G188" s="84"/>
+      <c r="F188" s="136">
+        <f>7/3.281</f>
+        <v>2.1334958854007922</v>
+      </c>
+      <c r="G188" s="84">
+        <f t="shared" si="22"/>
+        <v>-2.2759023465110548</v>
+      </c>
       <c r="H188" s="136"/>
       <c r="I188" s="136"/>
       <c r="J188" s="136"/>
@@ -13875,23 +13875,23 @@
     <row r="189" spans="1:11">
       <c r="A189" s="134"/>
       <c r="B189" s="142" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C189" s="135">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="D189" s="136">
-        <f>2*(15.5/3.281)+2*(13.083/3.281)</f>
-        <v>17.423346540688812</v>
+        <f>6/3.281</f>
+        <v>1.8287107589149649</v>
       </c>
       <c r="E189" s="136"/>
       <c r="F189" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
+        <f>4/3.281</f>
+        <v>1.2191405059433098</v>
       </c>
       <c r="G189" s="84">
-        <f t="shared" ref="G189" si="22">PRODUCT(C189:F189)</f>
-        <v>46.465797693089634</v>
+        <f t="shared" si="22"/>
+        <v>-4.4589107196951288</v>
       </c>
       <c r="H189" s="136"/>
       <c r="I189" s="136"/>
@@ -13900,23 +13900,22 @@
     </row>
     <row r="190" spans="1:11">
       <c r="A190" s="134"/>
-      <c r="B190" s="142" t="s">
-        <v>191</v>
-      </c>
+      <c r="B190" s="142"/>
       <c r="C190" s="135">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="D190" s="136">
-        <f>3.5/3.281</f>
-        <v>1.0667479427003961</v>
+        <f>4/3.281</f>
+        <v>1.2191405059433098</v>
       </c>
       <c r="E190" s="136"/>
       <c r="F190" s="136">
-        <v>2.1</v>
+        <f>4/3.281</f>
+        <v>1.2191405059433098</v>
       </c>
       <c r="G190" s="84">
-        <f t="shared" ref="G190:G192" si="23">PRODUCT(C190:F190)</f>
-        <v>-8.9606827186833282</v>
+        <f t="shared" si="22"/>
+        <v>-1.4863035732317094</v>
       </c>
       <c r="H190" s="136"/>
       <c r="I190" s="136"/>
@@ -13924,61 +13923,54 @@
       <c r="K190" s="137"/>
     </row>
     <row r="191" spans="1:11">
-      <c r="A191" s="134"/>
-      <c r="B191" s="142"/>
-      <c r="C191" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D191" s="136">
-        <v>0.75</v>
-      </c>
-      <c r="E191" s="136"/>
-      <c r="F191" s="136">
-        <v>1.8</v>
-      </c>
-      <c r="G191" s="84">
-        <f t="shared" si="23"/>
-        <v>-1.35</v>
-      </c>
-      <c r="H191" s="136"/>
-      <c r="I191" s="136"/>
-      <c r="J191" s="136"/>
-      <c r="K191" s="137"/>
+      <c r="A191" s="77"/>
+      <c r="B191" s="92"/>
+      <c r="C191" s="83"/>
+      <c r="D191" s="80"/>
+      <c r="E191" s="80"/>
+      <c r="F191" s="80"/>
+      <c r="G191" s="80">
+        <f>SUM(G186:G190)</f>
+        <v>23.410674687999336</v>
+      </c>
+      <c r="H191" s="80" t="s">
+        <v>23</v>
+      </c>
+      <c r="I191" s="80">
+        <f>1.15*60.3</f>
+        <v>69.344999999999985</v>
+      </c>
+      <c r="J191" s="80">
+        <f>G191*I191</f>
+        <v>1623.4132362393136</v>
+      </c>
+      <c r="K191" s="81"/>
     </row>
     <row r="192" spans="1:11">
       <c r="A192" s="134"/>
-      <c r="B192" s="142" t="s">
-        <v>192</v>
-      </c>
-      <c r="C192" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D192" s="136">
-        <v>0.9</v>
-      </c>
+      <c r="B192" s="133"/>
+      <c r="C192" s="135"/>
+      <c r="D192" s="136"/>
       <c r="E192" s="136"/>
-      <c r="F192" s="136">
-        <v>1.8</v>
-      </c>
-      <c r="G192" s="84">
-        <f t="shared" si="23"/>
-        <v>-1.62</v>
-      </c>
+      <c r="F192" s="136"/>
+      <c r="G192" s="136"/>
       <c r="H192" s="136"/>
       <c r="I192" s="136"/>
       <c r="J192" s="136"/>
       <c r="K192" s="137"/>
     </row>
-    <row r="193" spans="1:11">
-      <c r="A193" s="134"/>
-      <c r="B193" s="143" t="s">
-        <v>199</v>
+    <row r="193" spans="1:11" ht="45.75">
+      <c r="A193" s="134">
+        <v>21</v>
+      </c>
+      <c r="B193" s="115" t="s">
+        <v>206</v>
       </c>
       <c r="C193" s="135"/>
       <c r="D193" s="136"/>
       <c r="E193" s="136"/>
       <c r="F193" s="136"/>
-      <c r="G193" s="84"/>
+      <c r="G193" s="136"/>
       <c r="H193" s="136"/>
       <c r="I193" s="136"/>
       <c r="J193" s="136"/>
@@ -13986,25 +13978,14 @@
     </row>
     <row r="194" spans="1:11">
       <c r="A194" s="134"/>
-      <c r="B194" s="142" t="s">
-        <v>196</v>
-      </c>
-      <c r="C194" s="135">
-        <v>1</v>
-      </c>
-      <c r="D194" s="136">
-        <f>2*(10.5/3.281)+2*(13.5/3.281)</f>
-        <v>14.629686071319718</v>
-      </c>
+      <c r="B194" s="120" t="s">
+        <v>189</v>
+      </c>
+      <c r="C194" s="135"/>
+      <c r="D194" s="136"/>
       <c r="E194" s="136"/>
-      <c r="F194" s="136">
-        <f>8.75/3.281</f>
-        <v>2.6668698567509903</v>
-      </c>
-      <c r="G194" s="84">
-        <f t="shared" ref="G194:G198" si="24">PRODUCT(C194:F194)</f>
-        <v>39.015468797332375</v>
-      </c>
+      <c r="F194" s="136"/>
+      <c r="G194" s="136"/>
       <c r="H194" s="136"/>
       <c r="I194" s="136"/>
       <c r="J194" s="136"/>
@@ -14013,47 +13994,49 @@
     <row r="195" spans="1:11">
       <c r="A195" s="134"/>
       <c r="B195" s="142" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C195" s="135">
         <v>1</v>
       </c>
       <c r="D195" s="136">
-        <f>2*(10.917/3.281)+(13.17/3.281)</f>
-        <v>10.668698567509905</v>
+        <f>2*(28.25/3.281)+2*(13.42/3.281)</f>
+        <v>25.400792441328861</v>
       </c>
       <c r="E195" s="136"/>
       <c r="F195" s="136">
-        <f>8.667/3.281</f>
-        <v>2.6415726912526667</v>
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
       </c>
       <c r="G195" s="84">
-        <f t="shared" si="24"/>
-        <v>28.182142787140609</v>
+        <f t="shared" ref="G195:G202" si="23">PRODUCT(C195:F195)</f>
+        <v>67.74060769936834</v>
       </c>
       <c r="H195" s="136"/>
       <c r="I195" s="136"/>
       <c r="J195" s="136"/>
       <c r="K195" s="137"/>
     </row>
-    <row r="196" spans="1:11">
+    <row r="196" spans="1:11" ht="31.5">
       <c r="A196" s="134"/>
-      <c r="B196" s="142"/>
+      <c r="B196" s="142" t="s">
+        <v>193</v>
+      </c>
       <c r="C196" s="135">
         <v>1</v>
       </c>
       <c r="D196" s="136">
-        <f>(13.17/3.281)</f>
-        <v>4.0140201158183482</v>
-      </c>
-      <c r="E196" s="136">
-        <f>(10.917/3.281)</f>
-        <v>3.3273392258457783</v>
-      </c>
-      <c r="F196" s="136"/>
+        <f>2*(28.25/3.281)+2*(13.083/3.281)</f>
+        <v>25.195367266077415</v>
+      </c>
+      <c r="E196" s="136"/>
+      <c r="F196" s="136">
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
+      </c>
       <c r="G196" s="84">
-        <f t="shared" si="24"/>
-        <v>13.356006584696404</v>
+        <f t="shared" si="23"/>
+        <v>67.192765491672461</v>
       </c>
       <c r="H196" s="136"/>
       <c r="I196" s="136"/>
@@ -14063,21 +14046,22 @@
     <row r="197" spans="1:11">
       <c r="A197" s="134"/>
       <c r="B197" s="142" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="C197" s="135">
         <v>-1</v>
       </c>
       <c r="D197" s="136">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E197" s="136"/>
       <c r="F197" s="136">
-        <v>0.9</v>
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
       </c>
       <c r="G197" s="84">
-        <f t="shared" si="24"/>
-        <v>-1.35</v>
+        <f t="shared" si="23"/>
+        <v>-2.9259372142639433</v>
       </c>
       <c r="H197" s="136"/>
       <c r="I197" s="136"/>
@@ -14086,23 +14070,21 @@
     </row>
     <row r="198" spans="1:11">
       <c r="A198" s="134"/>
-      <c r="B198" s="142" t="s">
-        <v>191</v>
-      </c>
+      <c r="B198" s="142"/>
       <c r="C198" s="135">
         <v>-1</v>
       </c>
       <c r="D198" s="136">
-        <f>3.5/3.281</f>
+        <f t="shared" ref="D198" si="24">3.5/3.281</f>
         <v>1.0667479427003961</v>
       </c>
       <c r="E198" s="136"/>
       <c r="F198" s="136">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="G198" s="84">
-        <f t="shared" si="24"/>
-        <v>-1.920146296860713</v>
+        <f t="shared" ref="G198:G199" si="25">PRODUCT(C198:F198)</f>
+        <v>-2.2401706796708321</v>
       </c>
       <c r="H198" s="136"/>
       <c r="I198" s="136"/>
@@ -14111,23 +14093,20 @@
     </row>
     <row r="199" spans="1:11">
       <c r="A199" s="134"/>
-      <c r="B199" s="142" t="s">
-        <v>192</v>
-      </c>
+      <c r="B199" s="142"/>
       <c r="C199" s="135">
         <v>-1</v>
       </c>
       <c r="D199" s="136">
-        <v>1.8</v>
+        <v>0.75</v>
       </c>
       <c r="E199" s="136"/>
       <c r="F199" s="136">
-        <f>4.5/3.281</f>
-        <v>1.3715330691862238</v>
+        <v>1.8</v>
       </c>
       <c r="G199" s="84">
-        <f>PRODUCT(C199:F199)</f>
-        <v>-2.4687595245352028</v>
+        <f t="shared" si="25"/>
+        <v>-1.35</v>
       </c>
       <c r="H199" s="136"/>
       <c r="I199" s="136"/>
@@ -14135,54 +14114,68 @@
       <c r="K199" s="137"/>
     </row>
     <row r="200" spans="1:11">
-      <c r="A200" s="77"/>
-      <c r="B200" s="92"/>
-      <c r="C200" s="83"/>
-      <c r="D200" s="80"/>
-      <c r="E200" s="80"/>
-      <c r="F200" s="80"/>
-      <c r="G200" s="80">
-        <f>SUM(G180:G199)</f>
-        <v>221.74709261928581</v>
-      </c>
-      <c r="H200" s="80" t="s">
-        <v>23</v>
-      </c>
-      <c r="I200" s="80">
-        <f>1.15*125.5</f>
-        <v>144.32499999999999</v>
-      </c>
-      <c r="J200" s="80">
-        <f>G200*I200</f>
-        <v>32003.64914227842</v>
-      </c>
-      <c r="K200" s="81"/>
+      <c r="A200" s="134"/>
+      <c r="B200" s="142" t="s">
+        <v>188</v>
+      </c>
+      <c r="C200" s="135">
+        <v>-1</v>
+      </c>
+      <c r="D200" s="136">
+        <v>0.9</v>
+      </c>
+      <c r="E200" s="136"/>
+      <c r="F200" s="136">
+        <v>1.8</v>
+      </c>
+      <c r="G200" s="84">
+        <f t="shared" si="23"/>
+        <v>-1.62</v>
+      </c>
+      <c r="H200" s="136"/>
+      <c r="I200" s="136"/>
+      <c r="J200" s="136"/>
+      <c r="K200" s="137"/>
     </row>
     <row r="201" spans="1:11">
       <c r="A201" s="134"/>
-      <c r="B201" s="133"/>
-      <c r="C201" s="135"/>
-      <c r="D201" s="136"/>
+      <c r="B201" s="142"/>
+      <c r="C201" s="135">
+        <v>-6</v>
+      </c>
+      <c r="D201" s="136">
+        <v>1.8</v>
+      </c>
       <c r="E201" s="136"/>
-      <c r="F201" s="136"/>
-      <c r="G201" s="136"/>
+      <c r="F201" s="136">
+        <v>1.2</v>
+      </c>
+      <c r="G201" s="84">
+        <f t="shared" si="23"/>
+        <v>-12.96</v>
+      </c>
       <c r="H201" s="136"/>
       <c r="I201" s="136"/>
       <c r="J201" s="136"/>
       <c r="K201" s="137"/>
     </row>
-    <row r="202" spans="1:11" ht="30.75">
-      <c r="A202" s="134">
-        <v>22</v>
-      </c>
-      <c r="B202" s="115" t="s">
-        <v>202</v>
-      </c>
-      <c r="C202" s="135"/>
-      <c r="D202" s="136"/>
+    <row r="202" spans="1:11">
+      <c r="A202" s="134"/>
+      <c r="B202" s="142"/>
+      <c r="C202" s="135">
+        <v>-1</v>
+      </c>
+      <c r="D202" s="136">
+        <v>1.2</v>
+      </c>
       <c r="E202" s="136"/>
-      <c r="F202" s="136"/>
-      <c r="G202" s="136"/>
+      <c r="F202" s="136">
+        <v>1.2</v>
+      </c>
+      <c r="G202" s="84">
+        <f t="shared" si="23"/>
+        <v>-1.44</v>
+      </c>
       <c r="H202" s="136"/>
       <c r="I202" s="136"/>
       <c r="J202" s="136"/>
@@ -14191,13 +14184,13 @@
     <row r="203" spans="1:11">
       <c r="A203" s="134"/>
       <c r="B203" s="120" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C203" s="135"/>
       <c r="D203" s="136"/>
       <c r="E203" s="136"/>
       <c r="F203" s="136"/>
-      <c r="G203" s="136"/>
+      <c r="G203" s="84"/>
       <c r="H203" s="136"/>
       <c r="I203" s="136"/>
       <c r="J203" s="136"/>
@@ -14206,23 +14199,23 @@
     <row r="204" spans="1:11">
       <c r="A204" s="134"/>
       <c r="B204" s="142" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="C204" s="135">
         <v>1</v>
       </c>
       <c r="D204" s="136">
-        <f>2*(29.917/3.281)+2*(28.5/3.281)</f>
-        <v>35.609265467845169</v>
+        <f>2*(15.5/3.281)+2*(13.083/3.281)</f>
+        <v>17.423346540688812</v>
       </c>
       <c r="E204" s="136"/>
       <c r="F204" s="136">
-        <f>9.33/3.281</f>
-        <v>2.8436452301127706</v>
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
       </c>
       <c r="G204" s="84">
-        <f t="shared" ref="G204:G209" si="25">PRODUCT(C204:F204)</f>
-        <v>101.26011789545731</v>
+        <f t="shared" ref="G204" si="26">PRODUCT(C204:F204)</f>
+        <v>46.465797693089634</v>
       </c>
       <c r="H204" s="136"/>
       <c r="I204" s="136"/>
@@ -14232,22 +14225,22 @@
     <row r="205" spans="1:11">
       <c r="A205" s="134"/>
       <c r="B205" s="142" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C205" s="135">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="D205" s="136">
-        <v>1.2</v>
+        <f>3.5/3.281</f>
+        <v>1.0667479427003961</v>
       </c>
       <c r="E205" s="136"/>
       <c r="F205" s="136">
-        <f>8/3.281</f>
-        <v>2.4382810118866196</v>
+        <v>2.1</v>
       </c>
       <c r="G205" s="84">
-        <f t="shared" si="25"/>
-        <v>-2.9259372142639433</v>
+        <f t="shared" ref="G205:G207" si="27">PRODUCT(C205:F205)</f>
+        <v>-8.9606827186833282</v>
       </c>
       <c r="H205" s="136"/>
       <c r="I205" s="136"/>
@@ -14256,22 +14249,20 @@
     </row>
     <row r="206" spans="1:11">
       <c r="A206" s="134"/>
-      <c r="B206" s="142" t="s">
-        <v>192</v>
-      </c>
+      <c r="B206" s="142"/>
       <c r="C206" s="135">
         <v>-1</v>
       </c>
       <c r="D206" s="136">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="E206" s="136"/>
       <c r="F206" s="136">
         <v>1.8</v>
       </c>
       <c r="G206" s="84">
-        <f t="shared" si="25"/>
-        <v>-1.62</v>
+        <f t="shared" si="27"/>
+        <v>-1.35</v>
       </c>
       <c r="H206" s="136"/>
       <c r="I206" s="136"/>
@@ -14280,20 +14271,22 @@
     </row>
     <row r="207" spans="1:11">
       <c r="A207" s="134"/>
-      <c r="B207" s="142"/>
+      <c r="B207" s="142" t="s">
+        <v>188</v>
+      </c>
       <c r="C207" s="135">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="D207" s="136">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="E207" s="136"/>
       <c r="F207" s="136">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G207" s="84">
-        <f t="shared" si="25"/>
-        <v>-12.96</v>
+        <f t="shared" si="27"/>
+        <v>-1.62</v>
       </c>
       <c r="H207" s="136"/>
       <c r="I207" s="136"/>
@@ -14302,21 +14295,14 @@
     </row>
     <row r="208" spans="1:11">
       <c r="A208" s="134"/>
-      <c r="B208" s="142"/>
-      <c r="C208" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D208" s="136">
-        <v>1.2</v>
-      </c>
+      <c r="B208" s="143" t="s">
+        <v>194</v>
+      </c>
+      <c r="C208" s="135"/>
+      <c r="D208" s="136"/>
       <c r="E208" s="136"/>
-      <c r="F208" s="136">
-        <v>1.2</v>
-      </c>
-      <c r="G208" s="84">
-        <f t="shared" si="25"/>
-        <v>-1.44</v>
-      </c>
+      <c r="F208" s="136"/>
+      <c r="G208" s="84"/>
       <c r="H208" s="136"/>
       <c r="I208" s="136"/>
       <c r="J208" s="136"/>
@@ -14324,20 +14310,24 @@
     </row>
     <row r="209" spans="1:11">
       <c r="A209" s="134"/>
-      <c r="B209" s="142"/>
+      <c r="B209" s="142" t="s">
+        <v>191</v>
+      </c>
       <c r="C209" s="135">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D209" s="136">
-        <v>0.9</v>
+        <f>2*(10.5/3.281)+2*(13.5/3.281)</f>
+        <v>14.629686071319718</v>
       </c>
       <c r="E209" s="136"/>
       <c r="F209" s="136">
-        <v>1.2</v>
-      </c>
-      <c r="G209" s="139">
-        <f t="shared" si="25"/>
-        <v>-1.08</v>
+        <f>8.75/3.281</f>
+        <v>2.6668698567509903</v>
+      </c>
+      <c r="G209" s="84">
+        <f t="shared" ref="G209:G213" si="28">PRODUCT(C209:F209)</f>
+        <v>39.015468797332375</v>
       </c>
       <c r="H209" s="136"/>
       <c r="I209" s="136"/>
@@ -14346,14 +14336,25 @@
     </row>
     <row r="210" spans="1:11">
       <c r="A210" s="134"/>
-      <c r="B210" s="120" t="s">
-        <v>197</v>
-      </c>
-      <c r="C210" s="135"/>
-      <c r="D210" s="136"/>
+      <c r="B210" s="142" t="s">
+        <v>195</v>
+      </c>
+      <c r="C210" s="135">
+        <v>1</v>
+      </c>
+      <c r="D210" s="136">
+        <f>2*(10.917/3.281)+(13.17/3.281)</f>
+        <v>10.668698567509905</v>
+      </c>
       <c r="E210" s="136"/>
-      <c r="F210" s="136"/>
-      <c r="G210" s="84"/>
+      <c r="F210" s="136">
+        <f>8.667/3.281</f>
+        <v>2.6415726912526667</v>
+      </c>
+      <c r="G210" s="84">
+        <f t="shared" si="28"/>
+        <v>28.182142787140609</v>
+      </c>
       <c r="H210" s="136"/>
       <c r="I210" s="136"/>
       <c r="J210" s="136"/>
@@ -14361,24 +14362,22 @@
     </row>
     <row r="211" spans="1:11">
       <c r="A211" s="134"/>
-      <c r="B211" s="142" t="s">
-        <v>203</v>
-      </c>
+      <c r="B211" s="142"/>
       <c r="C211" s="135">
         <v>1</v>
       </c>
       <c r="D211" s="136">
-        <f>2*(29.917/3.281)+2*(28.5/3.281)</f>
-        <v>35.609265467845169</v>
-      </c>
-      <c r="E211" s="136"/>
-      <c r="F211" s="136">
-        <f>9.33/3.281</f>
-        <v>2.8436452301127706</v>
-      </c>
+        <f>(13.17/3.281)</f>
+        <v>4.0140201158183482</v>
+      </c>
+      <c r="E211" s="136">
+        <f>(10.917/3.281)</f>
+        <v>3.3273392258457783</v>
+      </c>
+      <c r="F211" s="136"/>
       <c r="G211" s="84">
-        <f t="shared" ref="G211" si="26">PRODUCT(C211:F211)</f>
-        <v>101.26011789545731</v>
+        <f t="shared" si="28"/>
+        <v>13.356006584696404</v>
       </c>
       <c r="H211" s="136"/>
       <c r="I211" s="136"/>
@@ -14388,22 +14387,21 @@
     <row r="212" spans="1:11">
       <c r="A212" s="134"/>
       <c r="B212" s="142" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C212" s="135">
         <v>-1</v>
       </c>
       <c r="D212" s="136">
-        <f>3.5/3.281</f>
-        <v>1.0667479427003961</v>
+        <v>1.5</v>
       </c>
       <c r="E212" s="136"/>
       <c r="F212" s="136">
-        <v>2.1</v>
+        <v>0.9</v>
       </c>
       <c r="G212" s="84">
-        <f t="shared" ref="G212:G216" si="27">PRODUCT(C212:F212)</f>
-        <v>-2.2401706796708321</v>
+        <f t="shared" si="28"/>
+        <v>-1.35</v>
       </c>
       <c r="H212" s="136"/>
       <c r="I212" s="136"/>
@@ -14413,21 +14411,22 @@
     <row r="213" spans="1:11">
       <c r="A213" s="134"/>
       <c r="B213" s="142" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C213" s="135">
         <v>-1</v>
       </c>
       <c r="D213" s="136">
-        <v>0.9</v>
+        <f>3.5/3.281</f>
+        <v>1.0667479427003961</v>
       </c>
       <c r="E213" s="136"/>
       <c r="F213" s="136">
         <v>1.8</v>
       </c>
       <c r="G213" s="84">
-        <f t="shared" si="27"/>
-        <v>-1.62</v>
+        <f t="shared" si="28"/>
+        <v>-1.920146296860713</v>
       </c>
       <c r="H213" s="136"/>
       <c r="I213" s="136"/>
@@ -14436,20 +14435,23 @@
     </row>
     <row r="214" spans="1:11">
       <c r="A214" s="134"/>
-      <c r="B214" s="142"/>
+      <c r="B214" s="142" t="s">
+        <v>188</v>
+      </c>
       <c r="C214" s="135">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="D214" s="136">
         <v>1.8</v>
       </c>
       <c r="E214" s="136"/>
       <c r="F214" s="136">
-        <v>1.2</v>
+        <f>4.5/3.281</f>
+        <v>1.3715330691862238</v>
       </c>
       <c r="G214" s="84">
-        <f t="shared" si="27"/>
-        <v>-12.96</v>
+        <f>PRODUCT(C214:F214)</f>
+        <v>-2.4687595245352028</v>
       </c>
       <c r="H214" s="136"/>
       <c r="I214" s="136"/>
@@ -14457,185 +14459,175 @@
       <c r="K214" s="137"/>
     </row>
     <row r="215" spans="1:11">
-      <c r="A215" s="134"/>
-      <c r="B215" s="142"/>
-      <c r="C215" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D215" s="136">
-        <v>1.2</v>
-      </c>
-      <c r="E215" s="136"/>
-      <c r="F215" s="136">
-        <v>1.2</v>
-      </c>
-      <c r="G215" s="84">
-        <f t="shared" si="27"/>
-        <v>-1.44</v>
-      </c>
-      <c r="H215" s="136"/>
-      <c r="I215" s="136"/>
-      <c r="J215" s="136"/>
-      <c r="K215" s="137"/>
+      <c r="A215" s="77"/>
+      <c r="B215" s="92"/>
+      <c r="C215" s="83"/>
+      <c r="D215" s="80"/>
+      <c r="E215" s="80"/>
+      <c r="F215" s="80"/>
+      <c r="G215" s="80">
+        <f>SUM(G195:G214)</f>
+        <v>221.74709261928581</v>
+      </c>
+      <c r="H215" s="80" t="s">
+        <v>23</v>
+      </c>
+      <c r="I215" s="80">
+        <f>1.15*195.14</f>
+        <v>224.41099999999997</v>
+      </c>
+      <c r="J215" s="80">
+        <f>G215*I215</f>
+        <v>49762.486801786545</v>
+      </c>
+      <c r="K215" s="81"/>
     </row>
     <row r="216" spans="1:11">
       <c r="A216" s="134"/>
-      <c r="B216" s="142"/>
-      <c r="C216" s="135">
-        <v>-1</v>
-      </c>
-      <c r="D216" s="136">
-        <v>0.9</v>
-      </c>
+      <c r="B216" s="133"/>
+      <c r="C216" s="135"/>
+      <c r="D216" s="136"/>
       <c r="E216" s="136"/>
-      <c r="F216" s="136">
-        <v>1.2</v>
-      </c>
-      <c r="G216" s="139">
-        <f t="shared" si="27"/>
-        <v>-1.08</v>
-      </c>
+      <c r="F216" s="136"/>
+      <c r="G216" s="136"/>
       <c r="H216" s="136"/>
       <c r="I216" s="136"/>
       <c r="J216" s="136"/>
       <c r="K216" s="137"/>
     </row>
-    <row r="217" spans="1:11">
-      <c r="A217" s="134"/>
-      <c r="B217" s="143" t="s">
-        <v>199</v>
-      </c>
-      <c r="C217" s="135"/>
-      <c r="D217" s="136"/>
-      <c r="E217" s="136"/>
-      <c r="F217" s="136"/>
-      <c r="G217" s="84"/>
-      <c r="H217" s="136"/>
-      <c r="I217" s="136"/>
-      <c r="J217" s="136"/>
-      <c r="K217" s="137"/>
+    <row r="217" spans="1:11" ht="31.5">
+      <c r="A217" s="77">
+        <v>22</v>
+      </c>
+      <c r="B217" s="120" t="s">
+        <v>141</v>
+      </c>
+      <c r="C217" s="83"/>
+      <c r="D217" s="80"/>
+      <c r="E217" s="80"/>
+      <c r="F217" s="80"/>
+      <c r="G217" s="80"/>
+      <c r="H217" s="80"/>
+      <c r="I217" s="80"/>
+      <c r="J217" s="80"/>
+      <c r="K217" s="81"/>
     </row>
     <row r="218" spans="1:11">
-      <c r="A218" s="134"/>
-      <c r="B218" s="142" t="s">
-        <v>204</v>
-      </c>
-      <c r="C218" s="135">
+      <c r="A218" s="77"/>
+      <c r="B218" s="94" t="s">
+        <v>142</v>
+      </c>
+      <c r="C218" s="83">
         <v>1</v>
       </c>
-      <c r="D218" s="136">
-        <f>(11.833/3.281)+(14.833/3.281)</f>
-        <v>8.1274001828710745</v>
-      </c>
-      <c r="E218" s="136"/>
-      <c r="F218" s="136">
-        <f>9.33/3.281</f>
-        <v>2.8436452301127706</v>
-      </c>
+      <c r="D218" s="80">
+        <f>0.9</f>
+        <v>0.9</v>
+      </c>
+      <c r="E218" s="80"/>
+      <c r="F218" s="80"/>
       <c r="G218" s="84">
-        <f t="shared" ref="G218" si="28">PRODUCT(C218:F218)</f>
-        <v>23.11144276323899</v>
-      </c>
-      <c r="H218" s="136"/>
-      <c r="I218" s="136"/>
-      <c r="J218" s="136"/>
-      <c r="K218" s="137"/>
+        <f t="shared" ref="G218:G220" si="29">PRODUCT(C218:F218)</f>
+        <v>0.9</v>
+      </c>
+      <c r="H218" s="80"/>
+      <c r="I218" s="80"/>
+      <c r="J218" s="80"/>
+      <c r="K218" s="81"/>
     </row>
     <row r="219" spans="1:11">
       <c r="A219" s="77"/>
-      <c r="B219" s="92"/>
-      <c r="C219" s="83"/>
-      <c r="D219" s="80"/>
+      <c r="B219" s="94" t="s">
+        <v>143</v>
+      </c>
+      <c r="C219" s="83">
+        <v>1</v>
+      </c>
+      <c r="D219" s="80">
+        <f>1.5</f>
+        <v>1.5</v>
+      </c>
       <c r="E219" s="80"/>
       <c r="F219" s="80"/>
-      <c r="G219" s="80">
-        <f>SUM(G204:G218)</f>
-        <v>186.26557066021883</v>
-      </c>
-      <c r="H219" s="80" t="s">
-        <v>23</v>
-      </c>
-      <c r="I219" s="80">
-        <f>1.15*192.85</f>
-        <v>221.77749999999997</v>
-      </c>
-      <c r="J219" s="80">
-        <f>G219*I219</f>
-        <v>41309.512597096676</v>
-      </c>
+      <c r="G219" s="84">
+        <f t="shared" si="29"/>
+        <v>1.5</v>
+      </c>
+      <c r="H219" s="80"/>
+      <c r="I219" s="80"/>
+      <c r="J219" s="80"/>
       <c r="K219" s="81"/>
     </row>
     <row r="220" spans="1:11">
-      <c r="A220" s="134"/>
-      <c r="B220" s="133"/>
-      <c r="C220" s="135"/>
-      <c r="D220" s="136"/>
-      <c r="E220" s="136"/>
-      <c r="F220" s="136"/>
-      <c r="G220" s="136"/>
-      <c r="H220" s="136"/>
-      <c r="I220" s="136"/>
-      <c r="J220" s="136"/>
-      <c r="K220" s="137"/>
-    </row>
-    <row r="221" spans="1:11" ht="31.5">
-      <c r="A221" s="77">
-        <v>23</v>
-      </c>
-      <c r="B221" s="120" t="s">
-        <v>141</v>
-      </c>
+      <c r="A220" s="77"/>
+      <c r="B220" s="94" t="s">
+        <v>144</v>
+      </c>
+      <c r="C220" s="83">
+        <v>2</v>
+      </c>
+      <c r="D220" s="80">
+        <v>0.9</v>
+      </c>
+      <c r="E220" s="80"/>
+      <c r="F220" s="80"/>
+      <c r="G220" s="84">
+        <f t="shared" si="29"/>
+        <v>1.8</v>
+      </c>
+      <c r="H220" s="80"/>
+      <c r="I220" s="80"/>
+      <c r="J220" s="80"/>
+      <c r="K220" s="81"/>
+    </row>
+    <row r="221" spans="1:11">
+      <c r="A221" s="77"/>
+      <c r="B221" s="92"/>
       <c r="C221" s="83"/>
       <c r="D221" s="80"/>
       <c r="E221" s="80"/>
       <c r="F221" s="80"/>
-      <c r="G221" s="80"/>
-      <c r="H221" s="80"/>
-      <c r="I221" s="80"/>
-      <c r="J221" s="80"/>
+      <c r="G221" s="80">
+        <f>SUM(G218:G220)</f>
+        <v>4.2</v>
+      </c>
+      <c r="H221" s="80" t="s">
+        <v>145</v>
+      </c>
+      <c r="I221" s="80">
+        <v>248</v>
+      </c>
+      <c r="J221" s="80">
+        <f>G221*I221</f>
+        <v>1041.6000000000001</v>
+      </c>
       <c r="K221" s="81"/>
     </row>
     <row r="222" spans="1:11">
       <c r="A222" s="77"/>
-      <c r="B222" s="94" t="s">
-        <v>142</v>
-      </c>
-      <c r="C222" s="83">
-        <v>1</v>
-      </c>
-      <c r="D222" s="80">
-        <f>0.9</f>
-        <v>0.9</v>
-      </c>
+      <c r="B222" s="92"/>
+      <c r="C222" s="83"/>
+      <c r="D222" s="80"/>
       <c r="E222" s="80"/>
       <c r="F222" s="80"/>
-      <c r="G222" s="84">
-        <f t="shared" ref="G222:G224" si="29">PRODUCT(C222:F222)</f>
-        <v>0.9</v>
-      </c>
+      <c r="G222" s="80"/>
       <c r="H222" s="80"/>
       <c r="I222" s="80"/>
       <c r="J222" s="80"/>
       <c r="K222" s="81"/>
     </row>
-    <row r="223" spans="1:11">
-      <c r="A223" s="77"/>
-      <c r="B223" s="94" t="s">
-        <v>143</v>
-      </c>
-      <c r="C223" s="83">
-        <v>1</v>
-      </c>
-      <c r="D223" s="80">
-        <f>1.5</f>
-        <v>1.5</v>
-      </c>
+    <row r="223" spans="1:11" ht="31.5">
+      <c r="A223" s="77">
+        <v>23</v>
+      </c>
+      <c r="B223" s="120" t="s">
+        <v>147</v>
+      </c>
+      <c r="C223" s="83"/>
+      <c r="D223" s="80"/>
       <c r="E223" s="80"/>
       <c r="F223" s="80"/>
-      <c r="G223" s="84">
-        <f t="shared" si="29"/>
-        <v>1.5</v>
-      </c>
+      <c r="G223" s="80"/>
       <c r="H223" s="80"/>
       <c r="I223" s="80"/>
       <c r="J223" s="80"/>
@@ -14644,19 +14636,19 @@
     <row r="224" spans="1:11">
       <c r="A224" s="77"/>
       <c r="B224" s="94" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C224" s="83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D224" s="80">
-        <v>0.9</v>
+        <v>9</v>
       </c>
       <c r="E224" s="80"/>
       <c r="F224" s="80"/>
       <c r="G224" s="84">
-        <f t="shared" si="29"/>
-        <v>1.8</v>
+        <f t="shared" ref="G224" si="30">PRODUCT(C224:F224)</f>
+        <v>9</v>
       </c>
       <c r="H224" s="80"/>
       <c r="I224" s="80"/>
@@ -14671,18 +14663,18 @@
       <c r="E225" s="80"/>
       <c r="F225" s="80"/>
       <c r="G225" s="80">
-        <f>SUM(G222:G224)</f>
-        <v>4.2</v>
+        <f>SUM(G224:G224)</f>
+        <v>9</v>
       </c>
       <c r="H225" s="80" t="s">
         <v>145</v>
       </c>
       <c r="I225" s="80">
-        <v>248</v>
+        <v>75</v>
       </c>
       <c r="J225" s="80">
         <f>G225*I225</f>
-        <v>1041.6000000000001</v>
+        <v>675</v>
       </c>
       <c r="K225" s="81"/>
     </row>
@@ -14699,12 +14691,12 @@
       <c r="J226" s="80"/>
       <c r="K226" s="81"/>
     </row>
-    <row r="227" spans="1:11" ht="31.5">
+    <row r="227" spans="1:11" ht="47.25">
       <c r="A227" s="77">
         <v>24</v>
       </c>
       <c r="B227" s="120" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C227" s="83"/>
       <c r="D227" s="80"/>
@@ -14724,14 +14716,12 @@
       <c r="C228" s="83">
         <v>1</v>
       </c>
-      <c r="D228" s="80">
-        <v>9</v>
-      </c>
+      <c r="D228" s="80"/>
       <c r="E228" s="80"/>
       <c r="F228" s="80"/>
       <c r="G228" s="84">
-        <f t="shared" ref="G228" si="30">PRODUCT(C228:F228)</f>
-        <v>9</v>
+        <f t="shared" ref="G228" si="31">PRODUCT(C228:F228)</f>
+        <v>1</v>
       </c>
       <c r="H228" s="80"/>
       <c r="I228" s="80"/>
@@ -14747,17 +14737,17 @@
       <c r="F229" s="80"/>
       <c r="G229" s="80">
         <f>SUM(G228:G228)</f>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H229" s="80" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="I229" s="80">
-        <v>75</v>
+        <v>1070</v>
       </c>
       <c r="J229" s="80">
         <f>G229*I229</f>
-        <v>675</v>
+        <v>1070</v>
       </c>
       <c r="K229" s="81"/>
     </row>
@@ -14774,12 +14764,12 @@
       <c r="J230" s="80"/>
       <c r="K230" s="81"/>
     </row>
-    <row r="231" spans="1:11" ht="47.25">
+    <row r="231" spans="1:11">
       <c r="A231" s="77">
         <v>25</v>
       </c>
       <c r="B231" s="120" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C231" s="83"/>
       <c r="D231" s="80"/>
@@ -14794,17 +14784,17 @@
     <row r="232" spans="1:11">
       <c r="A232" s="77"/>
       <c r="B232" s="94" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C232" s="83">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D232" s="80"/>
       <c r="E232" s="80"/>
       <c r="F232" s="80"/>
       <c r="G232" s="84">
-        <f t="shared" ref="G232" si="31">PRODUCT(C232:F232)</f>
-        <v>1</v>
+        <f t="shared" ref="G232" si="32">PRODUCT(C232:F232)</f>
+        <v>2</v>
       </c>
       <c r="H232" s="80"/>
       <c r="I232" s="80"/>
@@ -14820,17 +14810,17 @@
       <c r="F233" s="80"/>
       <c r="G233" s="80">
         <f>SUM(G232:G232)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H233" s="80" t="s">
         <v>149</v>
       </c>
       <c r="I233" s="80">
-        <v>1070</v>
+        <v>750</v>
       </c>
       <c r="J233" s="80">
         <f>G233*I233</f>
-        <v>1070</v>
+        <v>1500</v>
       </c>
       <c r="K233" s="81"/>
     </row>
@@ -14847,12 +14837,12 @@
       <c r="J234" s="80"/>
       <c r="K234" s="81"/>
     </row>
-    <row r="235" spans="1:11">
+    <row r="235" spans="1:11" ht="47.25">
       <c r="A235" s="77">
         <v>26</v>
       </c>
       <c r="B235" s="120" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
       <c r="C235" s="83"/>
       <c r="D235" s="80"/>
@@ -14867,17 +14857,17 @@
     <row r="236" spans="1:11">
       <c r="A236" s="77"/>
       <c r="B236" s="94" t="s">
-        <v>152</v>
+        <v>200</v>
       </c>
       <c r="C236" s="83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D236" s="80"/>
       <c r="E236" s="80"/>
       <c r="F236" s="80"/>
       <c r="G236" s="84">
-        <f t="shared" ref="G236" si="32">PRODUCT(C236:F236)</f>
-        <v>2</v>
+        <f t="shared" ref="G236" si="33">PRODUCT(C236:F236)</f>
+        <v>1</v>
       </c>
       <c r="H236" s="80"/>
       <c r="I236" s="80"/>
@@ -14893,17 +14883,17 @@
       <c r="F237" s="80"/>
       <c r="G237" s="80">
         <f>SUM(G236:G236)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H237" s="80" t="s">
         <v>149</v>
       </c>
       <c r="I237" s="80">
-        <v>750</v>
+        <v>8656</v>
       </c>
       <c r="J237" s="80">
         <f>G237*I237</f>
-        <v>1500</v>
+        <v>8656</v>
       </c>
       <c r="K237" s="81"/>
     </row>
@@ -14924,262 +14914,189 @@
       <c r="A239" s="77">
         <v>27</v>
       </c>
-      <c r="B239" s="120" t="s">
-        <v>205</v>
-      </c>
-      <c r="C239" s="83"/>
+      <c r="B239" s="93" t="s">
+        <v>207</v>
+      </c>
+      <c r="C239" s="83">
+        <v>1</v>
+      </c>
       <c r="D239" s="80"/>
       <c r="E239" s="80"/>
       <c r="F239" s="80"/>
-      <c r="G239" s="80"/>
-      <c r="H239" s="80"/>
-      <c r="I239" s="80"/>
-      <c r="J239" s="80"/>
+      <c r="G239" s="80">
+        <v>1</v>
+      </c>
+      <c r="H239" s="80" t="s">
+        <v>128</v>
+      </c>
+      <c r="I239" s="84">
+        <v>16500</v>
+      </c>
+      <c r="J239" s="84">
+        <f>G239*I239</f>
+        <v>16500</v>
+      </c>
       <c r="K239" s="81"/>
     </row>
     <row r="240" spans="1:11">
       <c r="A240" s="77"/>
-      <c r="B240" s="94" t="s">
-        <v>206</v>
-      </c>
-      <c r="C240" s="83">
-        <v>1</v>
-      </c>
+      <c r="B240" s="99"/>
+      <c r="C240" s="83"/>
       <c r="D240" s="80"/>
       <c r="E240" s="80"/>
-      <c r="F240" s="80"/>
-      <c r="G240" s="84">
-        <f t="shared" ref="G240" si="33">PRODUCT(C240:F240)</f>
+      <c r="F240" s="84"/>
+      <c r="G240" s="80"/>
+      <c r="H240" s="80"/>
+      <c r="I240" s="84"/>
+      <c r="J240" s="84"/>
+      <c r="K240" s="81"/>
+    </row>
+    <row r="241" spans="1:11" ht="33" customHeight="1">
+      <c r="A241" s="77">
+        <v>28</v>
+      </c>
+      <c r="B241" s="93" t="s">
+        <v>75</v>
+      </c>
+      <c r="C241" s="83">
         <v>1</v>
       </c>
-      <c r="H240" s="80"/>
-      <c r="I240" s="80"/>
-      <c r="J240" s="80"/>
-      <c r="K240" s="81"/>
-    </row>
-    <row r="241" spans="1:11">
-      <c r="A241" s="77"/>
-      <c r="B241" s="92"/>
-      <c r="C241" s="83"/>
       <c r="D241" s="80"/>
       <c r="E241" s="80"/>
       <c r="F241" s="80"/>
       <c r="G241" s="80">
-        <f>SUM(G240:G240)</f>
         <v>1</v>
       </c>
       <c r="H241" s="80" t="s">
-        <v>149</v>
-      </c>
-      <c r="I241" s="80">
-        <v>8656</v>
-      </c>
-      <c r="J241" s="80">
+        <v>33</v>
+      </c>
+      <c r="I241" s="84">
+        <v>500</v>
+      </c>
+      <c r="J241" s="84">
         <f>G241*I241</f>
-        <v>8656</v>
+        <v>500</v>
       </c>
       <c r="K241" s="81"/>
     </row>
     <row r="242" spans="1:11">
-      <c r="A242" s="77"/>
-      <c r="B242" s="92"/>
-      <c r="C242" s="83"/>
-      <c r="D242" s="80"/>
-      <c r="E242" s="80"/>
-      <c r="F242" s="80"/>
-      <c r="G242" s="80"/>
+      <c r="A242" s="100"/>
+      <c r="B242" s="101"/>
+      <c r="C242" s="80"/>
+      <c r="D242" s="84"/>
+      <c r="E242" s="84"/>
+      <c r="F242" s="84"/>
+      <c r="G242" s="84"/>
       <c r="H242" s="80"/>
-      <c r="I242" s="80"/>
-      <c r="J242" s="80"/>
-      <c r="K242" s="81"/>
-    </row>
-    <row r="243" spans="1:11" ht="47.25" customHeight="1">
-      <c r="A243" s="77">
-        <v>28</v>
-      </c>
-      <c r="B243" s="93" t="s">
-        <v>179</v>
-      </c>
-      <c r="C243" s="83">
-        <v>1</v>
-      </c>
-      <c r="D243" s="80"/>
-      <c r="E243" s="80"/>
-      <c r="F243" s="80"/>
-      <c r="G243" s="80">
-        <v>1</v>
-      </c>
-      <c r="H243" s="80" t="s">
-        <v>128</v>
-      </c>
-      <c r="I243" s="84">
-        <v>45000</v>
-      </c>
-      <c r="J243" s="84">
-        <f>G243*I243</f>
-        <v>45000</v>
-      </c>
-      <c r="K243" s="81"/>
+      <c r="I242" s="84"/>
+      <c r="J242" s="102">
+        <f>SUM(J12:J241)</f>
+        <v>884738.59404214984</v>
+      </c>
+      <c r="K242" s="103"/>
+    </row>
+    <row r="243" spans="1:11">
+      <c r="A243" s="104"/>
+      <c r="B243" s="105"/>
+      <c r="C243" s="65"/>
+      <c r="D243" s="65"/>
+      <c r="E243" s="65"/>
+      <c r="F243" s="65"/>
+      <c r="G243" s="65"/>
+      <c r="H243" s="65"/>
+      <c r="I243" s="65"/>
+      <c r="J243" s="106"/>
+      <c r="K243" s="107"/>
     </row>
     <row r="244" spans="1:11">
-      <c r="A244" s="77"/>
-      <c r="B244" s="99"/>
-      <c r="C244" s="83"/>
-      <c r="D244" s="80"/>
-      <c r="E244" s="80"/>
-      <c r="F244" s="84"/>
-      <c r="G244" s="80"/>
-      <c r="H244" s="80"/>
-      <c r="I244" s="84"/>
-      <c r="J244" s="84"/>
-      <c r="K244" s="81"/>
-    </row>
-    <row r="245" spans="1:11" ht="33" customHeight="1">
-      <c r="A245" s="77">
-        <v>29</v>
-      </c>
-      <c r="B245" s="93" t="s">
-        <v>75</v>
-      </c>
-      <c r="C245" s="83">
-        <v>1</v>
-      </c>
-      <c r="D245" s="80"/>
-      <c r="E245" s="80"/>
-      <c r="F245" s="80"/>
-      <c r="G245" s="80">
-        <v>1</v>
-      </c>
-      <c r="H245" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="I245" s="84">
-        <v>500</v>
-      </c>
-      <c r="J245" s="84">
-        <f>G245*I245</f>
-        <v>500</v>
-      </c>
-      <c r="K245" s="81"/>
+      <c r="A244" s="104"/>
+      <c r="B244" s="75" t="s">
+        <v>12</v>
+      </c>
+      <c r="C244" s="144" t="s">
+        <v>66</v>
+      </c>
+      <c r="D244" s="144"/>
+      <c r="E244" s="75" t="s">
+        <v>67</v>
+      </c>
+      <c r="F244" s="108"/>
+      <c r="G244" s="109"/>
+      <c r="H244" s="108"/>
+      <c r="I244" s="109"/>
+      <c r="J244" s="108"/>
+      <c r="K244" s="108"/>
+    </row>
+    <row r="245" spans="1:11">
+      <c r="A245" s="104"/>
+      <c r="B245" s="79" t="s">
+        <v>13</v>
+      </c>
+      <c r="C245" s="145">
+        <f>+J242</f>
+        <v>884738.59404214984</v>
+      </c>
+      <c r="D245" s="145"/>
+      <c r="E245" s="110"/>
+      <c r="F245" s="108"/>
+      <c r="G245" s="111"/>
+      <c r="H245" s="108"/>
+      <c r="I245" s="109"/>
+      <c r="J245" s="108"/>
+      <c r="K245" s="108"/>
     </row>
     <row r="246" spans="1:11">
-      <c r="A246" s="100"/>
-      <c r="B246" s="101"/>
-      <c r="C246" s="80"/>
-      <c r="D246" s="84"/>
-      <c r="E246" s="84"/>
-      <c r="F246" s="84"/>
-      <c r="G246" s="84"/>
-      <c r="H246" s="80"/>
-      <c r="I246" s="84"/>
-      <c r="J246" s="102">
-        <f>SUM(J12:J245)</f>
-        <v>883372.89061096346</v>
-      </c>
-      <c r="K246" s="103"/>
+      <c r="A246" s="104"/>
+      <c r="B246" s="79" t="s">
+        <v>201</v>
+      </c>
+      <c r="C246" s="146">
+        <f>C245*13%</f>
+        <v>115016.01722547949</v>
+      </c>
+      <c r="D246" s="147"/>
+      <c r="E246" s="110"/>
+      <c r="F246" s="108"/>
+      <c r="G246" s="111"/>
+      <c r="H246" s="108"/>
+      <c r="I246" s="109"/>
+      <c r="J246" s="108"/>
+      <c r="K246" s="108"/>
     </row>
     <row r="247" spans="1:11">
       <c r="A247" s="104"/>
-      <c r="B247" s="105"/>
-      <c r="C247" s="65"/>
-      <c r="D247" s="65"/>
-      <c r="E247" s="65"/>
-      <c r="F247" s="65"/>
-      <c r="G247" s="65"/>
-      <c r="H247" s="65"/>
-      <c r="I247" s="65"/>
-      <c r="J247" s="106"/>
-      <c r="K247" s="107"/>
+      <c r="B247" s="79" t="s">
+        <v>202</v>
+      </c>
+      <c r="C247" s="146">
+        <f>SUM(C245:D246)</f>
+        <v>999754.61126762931</v>
+      </c>
+      <c r="D247" s="147"/>
+      <c r="E247" s="110"/>
+      <c r="F247" s="108"/>
+      <c r="G247" s="111"/>
+      <c r="H247" s="108"/>
+      <c r="I247" s="109"/>
+      <c r="J247" s="108"/>
+      <c r="K247" s="108"/>
     </row>
     <row r="248" spans="1:11">
-      <c r="A248" s="104"/>
-      <c r="B248" s="75" t="s">
-        <v>12</v>
-      </c>
-      <c r="C248" s="151" t="s">
-        <v>66</v>
-      </c>
-      <c r="D248" s="151"/>
-      <c r="E248" s="75" t="s">
-        <v>67</v>
-      </c>
-      <c r="F248" s="108"/>
-      <c r="G248" s="109"/>
-      <c r="H248" s="108"/>
-      <c r="I248" s="109"/>
-      <c r="J248" s="108"/>
-      <c r="K248" s="108"/>
-    </row>
-    <row r="249" spans="1:11">
-      <c r="A249" s="104"/>
-      <c r="B249" s="79" t="s">
-        <v>13</v>
-      </c>
-      <c r="C249" s="152">
-        <f>+J246</f>
-        <v>883372.89061096346</v>
-      </c>
-      <c r="D249" s="152"/>
-      <c r="E249" s="110"/>
-      <c r="F249" s="108"/>
-      <c r="G249" s="111"/>
-      <c r="H249" s="108"/>
-      <c r="I249" s="109"/>
-      <c r="J249" s="108"/>
-      <c r="K249" s="108"/>
-    </row>
-    <row r="250" spans="1:11">
-      <c r="A250" s="104"/>
-      <c r="B250" s="79" t="s">
-        <v>207</v>
-      </c>
-      <c r="C250" s="180">
-        <f>C249*13%</f>
-        <v>114838.47577942525</v>
-      </c>
-      <c r="D250" s="181"/>
-      <c r="E250" s="110"/>
-      <c r="F250" s="108"/>
-      <c r="G250" s="111"/>
-      <c r="H250" s="108"/>
-      <c r="I250" s="109"/>
-      <c r="J250" s="108"/>
-      <c r="K250" s="108"/>
-    </row>
-    <row r="251" spans="1:11">
-      <c r="A251" s="104"/>
-      <c r="B251" s="79" t="s">
-        <v>208</v>
-      </c>
-      <c r="C251" s="180">
-        <f>SUM(C249:D250)</f>
-        <v>998211.36639038869</v>
-      </c>
-      <c r="D251" s="181"/>
-      <c r="E251" s="110"/>
-      <c r="F251" s="108"/>
-      <c r="G251" s="111"/>
-      <c r="H251" s="108"/>
-      <c r="I251" s="109"/>
-      <c r="J251" s="108"/>
-      <c r="K251" s="108"/>
-    </row>
-    <row r="252" spans="1:11">
-      <c r="F252" s="37"/>
+      <c r="F248" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C248:D248"/>
-    <mergeCell ref="C249:D249"/>
-    <mergeCell ref="C250:D250"/>
-    <mergeCell ref="C251:D251"/>
-    <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="J5:K5"/>
+    <mergeCell ref="C244:D244"/>
+    <mergeCell ref="C245:D245"/>
+    <mergeCell ref="C246:D246"/>
+    <mergeCell ref="C247:D247"/>
+    <mergeCell ref="A6:F6"/>
   </mergeCells>
   <phoneticPr fontId="83" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>